<commit_message>
updated bycatch glossary with gear types
</commit_message>
<xml_diff>
--- a/data-raw/texts.xlsx
+++ b/data-raw/texts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub_2023\fisheriesXplorer\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26A487D9-2DDD-4C63-B91B-4023BC05F690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523558E1-3178-4680-8AE7-AA5F361413F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="826" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="826" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="glossary" sheetId="17" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="932">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1250" uniqueCount="998">
   <si>
     <t>section</t>
   </si>
@@ -4522,6 +4522,204 @@
   </si>
   <si>
     <t>Metier / fleet grouping</t>
+  </si>
+  <si>
+    <t>GTR</t>
+  </si>
+  <si>
+    <t>Trammel nets</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=45a8983a-2a25-4959-a5aa-eb15816ddfe0</t>
+  </si>
+  <si>
+    <t>LLD</t>
+  </si>
+  <si>
+    <t>Drifting longlines</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=327a2e44-ed48-44b0-900d-a07b4ac6e0fb</t>
+  </si>
+  <si>
+    <t>OTB</t>
+  </si>
+  <si>
+    <t>Bottom otter trawl</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=573c31dc-b343-42c2-9697-c9a20cfc6be0</t>
+  </si>
+  <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>Purse seine</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=68ca65b7-3374-4fec-8bdd-8a3ccd36d7a4</t>
+  </si>
+  <si>
+    <t>PTM</t>
+  </si>
+  <si>
+    <t>Pelagic pair trawl</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=8ce860fd-b3ea-4361-ad13-44a9f8535731</t>
+  </si>
+  <si>
+    <t>GNS</t>
+  </si>
+  <si>
+    <t>Set gillnet</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=55f84dad-e861-4d12-8582-b0fe00d99633</t>
+  </si>
+  <si>
+    <t>LLS</t>
+  </si>
+  <si>
+    <t>Set longlines</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=940eecd0-d03c-444c-b388-e01d0b72ac03</t>
+  </si>
+  <si>
+    <t>FPO</t>
+  </si>
+  <si>
+    <t>Pots and traps</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=fe1fbee6-5d67-439f-aabf-ca13c48a7d62</t>
+  </si>
+  <si>
+    <t>LHP</t>
+  </si>
+  <si>
+    <t>Hand and pole lines (hand-operated)</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=3e577955-36e8-41af-aef8-3c3e57b55327</t>
+  </si>
+  <si>
+    <t>FPN</t>
+  </si>
+  <si>
+    <t>Stationary uncovered pound nets</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=f94b5577-2827-45d8-8636-c5d6f7ba1926</t>
+  </si>
+  <si>
+    <t>FYK</t>
+  </si>
+  <si>
+    <t>Fyke nets</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=0a9f8e7e-9103-4e10-9feb-cc1ebf270996</t>
+  </si>
+  <si>
+    <t>OTM</t>
+  </si>
+  <si>
+    <t>Midwater otter trawl</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=4a7fcf3a-7bc2-4bcc-aa17-c5404761f48c</t>
+  </si>
+  <si>
+    <t>SDN</t>
+  </si>
+  <si>
+    <t>Anchored seine</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=9eded55c-2735-4d92-b9c5-97e7906b7de8</t>
+  </si>
+  <si>
+    <t>OTT</t>
+  </si>
+  <si>
+    <t>Milti-rig otter trawl</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=15d29f27-abbf-468c-8964-a481ea2958f3</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>Driftnet</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=2c822a11-cd1c-4dec-b693-2b01a19871f7</t>
+  </si>
+  <si>
+    <t>GTN</t>
+  </si>
+  <si>
+    <t>Gillnets-trammel nets</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=6f3c7b15-f8c1-4349-93d2-46a52a965beb</t>
+  </si>
+  <si>
+    <t>LTL</t>
+  </si>
+  <si>
+    <t>Trolling lines</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=8a4cbe19-220e-46c9-b59b-28719b32c3de</t>
+  </si>
+  <si>
+    <t>PTB</t>
+  </si>
+  <si>
+    <t>Bottom pair trawl</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=2d47bbb8-5ff8-4ae5-b94d-d151fc7ef509</t>
+  </si>
+  <si>
+    <t>TBB</t>
+  </si>
+  <si>
+    <t>Beam trawl</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=023236fc-b701-40b1-90d5-4d09ff60764c</t>
+  </si>
+  <si>
+    <t>SSC</t>
+  </si>
+  <si>
+    <t>Fly shooting seine</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=eb47154a-85a4-470a-afab-283eb769a5ec</t>
+  </si>
+  <si>
+    <t>DRB</t>
+  </si>
+  <si>
+    <t>Boat dredge</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=6028000e-4925-4313-90ef-1ab2461d8234</t>
+  </si>
+  <si>
+    <t>LHM</t>
+  </si>
+  <si>
+    <t>Hand and pole lines</t>
+  </si>
+  <si>
+    <t>https://vocab.ices.dk/?codeguid=30d806c1-550a-4d44-9e5d-e7887407e068</t>
   </si>
 </sst>
 </file>
@@ -4624,7 +4822,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4650,6 +4848,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4955,7 +5156,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF5EC4FE-E411-4E36-B8C3-47DB4028DB0F}">
-  <dimension ref="A1:C293"/>
+  <dimension ref="A1:C315"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.36328125" bestFit="1" customWidth="1"/>
@@ -5021,3179 +5222,3421 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>64</v>
+      <c r="A6" s="13" t="s">
+        <v>992</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>993</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>994</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>17</v>
+      <c r="A11" s="13" t="s">
+        <v>959</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>960</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>961</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>62</v>
+      <c r="A12" s="13" t="s">
+        <v>953</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>954</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>955</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>55</v>
+      <c r="A13" s="13" t="s">
+        <v>962</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>963</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>964</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>59</v>
+      <c r="A14" s="13" t="s">
+        <v>974</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>975</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>976</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
-        <v>931</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>59</v>
+      <c r="A15" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>948</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>949</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>57</v>
+      <c r="A16" s="13" t="s">
+        <v>977</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>978</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>979</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>56</v>
+      <c r="A17" s="13" t="s">
+        <v>932</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>933</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>934</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="13" t="s">
+        <v>995</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>996</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="13" t="s">
+        <v>956</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>957</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>935</v>
+      </c>
+      <c r="B22" t="s">
+        <v>936</v>
+      </c>
+      <c r="C22" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>950</v>
+      </c>
+      <c r="B23" t="s">
+        <v>951</v>
+      </c>
+      <c r="C23" t="s">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>980</v>
+      </c>
+      <c r="B25" t="s">
+        <v>981</v>
+      </c>
+      <c r="C25" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="14" t="s">
+        <v>931</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>938</v>
+      </c>
+      <c r="B31" t="s">
+        <v>939</v>
+      </c>
+      <c r="C31" t="s">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>965</v>
+      </c>
+      <c r="B32" t="s">
+        <v>966</v>
+      </c>
+      <c r="C32" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>971</v>
+      </c>
+      <c r="B33" t="s">
+        <v>972</v>
+      </c>
+      <c r="C33" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>941</v>
+      </c>
+      <c r="B34" t="s">
+        <v>942</v>
+      </c>
+      <c r="C34" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>983</v>
+      </c>
+      <c r="B35" t="s">
+        <v>984</v>
+      </c>
+      <c r="C35" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>944</v>
+      </c>
+      <c r="B36" t="s">
+        <v>945</v>
+      </c>
+      <c r="C36" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>968</v>
+      </c>
+      <c r="B37" t="s">
+        <v>969</v>
+      </c>
+      <c r="C37" t="s">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>989</v>
+      </c>
+      <c r="B38" t="s">
+        <v>990</v>
+      </c>
+      <c r="C38" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>986</v>
+      </c>
+      <c r="B40" t="s">
+        <v>987</v>
+      </c>
+      <c r="C40" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B41" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C41" s="15" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="8" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B42" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C42" s="15" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" s="8" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B43" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C43" s="15" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A25" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A27" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="B27" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="C27" s="10" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="C28" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="C29" s="10" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A30" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="C30" s="10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A31" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A32" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="C32" s="10" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="C33" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A34" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A35" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A36" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B36" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C36" s="10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="C37" s="10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A38" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="C38" s="11" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A39" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="C39" s="10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="B40" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="C40" s="10" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A41" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B41" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="C41" s="10" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A43" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="C43" s="10" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="10" t="s">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>133</v>
+        <v>67</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>134</v>
+        <v>68</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="s">
-        <v>135</v>
+        <v>69</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>136</v>
+        <v>70</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>137</v>
+        <v>71</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="10" t="s">
-        <v>138</v>
+        <v>72</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>139</v>
+        <v>73</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>140</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
-        <v>141</v>
+        <v>75</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>142</v>
+        <v>76</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>143</v>
+        <v>77</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="10" t="s">
-        <v>144</v>
+        <v>78</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>145</v>
+        <v>79</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="10" t="s">
-        <v>147</v>
+        <v>81</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>148</v>
+        <v>82</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>149</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="10" t="s">
-        <v>150</v>
+        <v>84</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>151</v>
+        <v>85</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>152</v>
+        <v>86</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="10" t="s">
-        <v>153</v>
+        <v>87</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>154</v>
+        <v>88</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>155</v>
+        <v>89</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="10" t="s">
-        <v>156</v>
+        <v>90</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>157</v>
+        <v>91</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>158</v>
+        <v>92</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="10" t="s">
-        <v>159</v>
+        <v>93</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>160</v>
+        <v>94</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>161</v>
+        <v>95</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="10" t="s">
-        <v>162</v>
+        <v>96</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>163</v>
+        <v>97</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>164</v>
+        <v>98</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="10" t="s">
-        <v>165</v>
+        <v>99</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>166</v>
+        <v>100</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>167</v>
+        <v>101</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="10" t="s">
-        <v>168</v>
+        <v>102</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>169</v>
+        <v>103</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>170</v>
+        <v>104</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
-        <v>171</v>
+        <v>105</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>172</v>
+        <v>106</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>173</v>
+        <v>107</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="10" t="s">
-        <v>174</v>
+        <v>108</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>175</v>
+        <v>109</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>176</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="10" t="s">
-        <v>177</v>
+        <v>111</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>178</v>
+        <v>112</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>179</v>
+        <v>113</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="10" t="s">
-        <v>180</v>
+        <v>114</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="C60" s="10" t="s">
-        <v>182</v>
+        <v>115</v>
+      </c>
+      <c r="C60" s="11" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="10" t="s">
-        <v>183</v>
+        <v>117</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>184</v>
+        <v>118</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>185</v>
+        <v>119</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="10" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>187</v>
+        <v>121</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>188</v>
+        <v>122</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="10" t="s">
-        <v>189</v>
+        <v>123</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>190</v>
+        <v>124</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>191</v>
+        <v>125</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="10" t="s">
-        <v>192</v>
+        <v>126</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>193</v>
+        <v>127</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>194</v>
+        <v>128</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" s="10" t="s">
-        <v>195</v>
+        <v>129</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>196</v>
+        <v>130</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>197</v>
+        <v>131</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" s="10" t="s">
-        <v>198</v>
+        <v>132</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>199</v>
+        <v>133</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>200</v>
+        <v>134</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" s="10" t="s">
-        <v>201</v>
+        <v>135</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>202</v>
+        <v>136</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>203</v>
+        <v>137</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" s="10" t="s">
-        <v>204</v>
+        <v>138</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>205</v>
+        <v>139</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>206</v>
+        <v>140</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" s="10" t="s">
-        <v>207</v>
+        <v>141</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>208</v>
+        <v>142</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>209</v>
+        <v>143</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" s="10" t="s">
-        <v>210</v>
+        <v>144</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>211</v>
+        <v>145</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>212</v>
+        <v>146</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" s="10" t="s">
-        <v>213</v>
+        <v>147</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>214</v>
+        <v>148</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>215</v>
+        <v>149</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" s="10" t="s">
-        <v>216</v>
+        <v>150</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>217</v>
+        <v>151</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>218</v>
+        <v>152</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" s="10" t="s">
-        <v>219</v>
+        <v>153</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>220</v>
+        <v>154</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>221</v>
+        <v>155</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" s="10" t="s">
-        <v>222</v>
+        <v>156</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>223</v>
+        <v>157</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>224</v>
+        <v>158</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" s="10" t="s">
-        <v>225</v>
+        <v>159</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>226</v>
+        <v>160</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>227</v>
+        <v>161</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" s="10" t="s">
-        <v>228</v>
+        <v>162</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>229</v>
+        <v>163</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>230</v>
+        <v>164</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" s="10" t="s">
-        <v>231</v>
+        <v>165</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>232</v>
+        <v>166</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>233</v>
+        <v>167</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" s="10" t="s">
-        <v>234</v>
+        <v>168</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>235</v>
+        <v>169</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>236</v>
+        <v>170</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" s="10" t="s">
-        <v>237</v>
+        <v>171</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>238</v>
+        <v>172</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>239</v>
+        <v>173</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" s="10" t="s">
-        <v>240</v>
+        <v>174</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>241</v>
+        <v>175</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" s="10" t="s">
-        <v>243</v>
+        <v>177</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>244</v>
+        <v>178</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>245</v>
+        <v>179</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" s="10" t="s">
-        <v>246</v>
+        <v>180</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>247</v>
+        <v>181</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>248</v>
+        <v>182</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" s="10" t="s">
-        <v>249</v>
+        <v>183</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>250</v>
+        <v>184</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>251</v>
+        <v>185</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" s="10" t="s">
-        <v>252</v>
+        <v>186</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>253</v>
+        <v>187</v>
       </c>
       <c r="C84" s="10" t="s">
-        <v>254</v>
+        <v>188</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" s="10" t="s">
-        <v>255</v>
+        <v>189</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>256</v>
+        <v>190</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>257</v>
+        <v>191</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A86" s="10" t="s">
-        <v>258</v>
+        <v>192</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>259</v>
+        <v>193</v>
       </c>
       <c r="C86" s="10" t="s">
-        <v>260</v>
+        <v>194</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" s="10" t="s">
-        <v>261</v>
+        <v>195</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>262</v>
+        <v>196</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>263</v>
+        <v>197</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" s="10" t="s">
-        <v>264</v>
+        <v>198</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>265</v>
+        <v>199</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>266</v>
+        <v>200</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" s="10" t="s">
-        <v>267</v>
+        <v>201</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>268</v>
+        <v>202</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>269</v>
+        <v>203</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" s="10" t="s">
-        <v>270</v>
+        <v>204</v>
       </c>
       <c r="B90" s="10" t="s">
-        <v>271</v>
+        <v>205</v>
       </c>
       <c r="C90" s="10" t="s">
-        <v>272</v>
+        <v>206</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" s="10" t="s">
-        <v>273</v>
+        <v>207</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>274</v>
+        <v>208</v>
       </c>
       <c r="C91" s="10" t="s">
-        <v>275</v>
+        <v>209</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" s="10" t="s">
-        <v>276</v>
+        <v>210</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>277</v>
+        <v>211</v>
       </c>
       <c r="C92" s="10" t="s">
-        <v>278</v>
+        <v>212</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" s="10" t="s">
-        <v>279</v>
+        <v>213</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>280</v>
+        <v>214</v>
       </c>
       <c r="C93" s="10" t="s">
-        <v>281</v>
+        <v>215</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" s="10" t="s">
-        <v>282</v>
+        <v>216</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>283</v>
+        <v>217</v>
       </c>
       <c r="C94" s="10" t="s">
-        <v>284</v>
+        <v>218</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A95" s="10" t="s">
-        <v>285</v>
+        <v>219</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>286</v>
+        <v>220</v>
       </c>
       <c r="C95" s="10" t="s">
-        <v>287</v>
+        <v>221</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A96" s="10" t="s">
-        <v>288</v>
+        <v>222</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>289</v>
+        <v>223</v>
       </c>
       <c r="C96" s="10" t="s">
-        <v>290</v>
+        <v>224</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A97" s="10" t="s">
-        <v>291</v>
+        <v>225</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>292</v>
+        <v>226</v>
       </c>
       <c r="C97" s="10" t="s">
-        <v>293</v>
+        <v>227</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A98" s="10" t="s">
-        <v>294</v>
+        <v>228</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>295</v>
+        <v>229</v>
       </c>
       <c r="C98" s="10" t="s">
-        <v>296</v>
+        <v>230</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A99" s="10" t="s">
-        <v>297</v>
+        <v>231</v>
       </c>
       <c r="B99" s="10" t="s">
-        <v>298</v>
+        <v>232</v>
       </c>
       <c r="C99" s="10" t="s">
-        <v>299</v>
+        <v>233</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A100" s="10" t="s">
-        <v>300</v>
+        <v>234</v>
       </c>
       <c r="B100" s="10" t="s">
-        <v>301</v>
+        <v>235</v>
       </c>
       <c r="C100" s="10" t="s">
-        <v>302</v>
+        <v>236</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A101" s="10" t="s">
-        <v>303</v>
+        <v>237</v>
       </c>
       <c r="B101" s="10" t="s">
-        <v>304</v>
+        <v>238</v>
       </c>
       <c r="C101" s="10" t="s">
-        <v>305</v>
+        <v>239</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A102" s="10" t="s">
-        <v>306</v>
+        <v>240</v>
       </c>
       <c r="B102" s="10" t="s">
-        <v>307</v>
+        <v>241</v>
       </c>
       <c r="C102" s="10" t="s">
-        <v>308</v>
+        <v>242</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A103" s="10" t="s">
-        <v>309</v>
+        <v>243</v>
       </c>
       <c r="B103" s="10" t="s">
-        <v>310</v>
+        <v>244</v>
       </c>
       <c r="C103" s="10" t="s">
-        <v>311</v>
+        <v>245</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A104" s="10" t="s">
-        <v>312</v>
+        <v>246</v>
       </c>
       <c r="B104" s="10" t="s">
-        <v>313</v>
+        <v>247</v>
       </c>
       <c r="C104" s="10" t="s">
-        <v>314</v>
+        <v>248</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A105" s="10" t="s">
-        <v>315</v>
+        <v>249</v>
       </c>
       <c r="B105" s="10" t="s">
-        <v>316</v>
+        <v>250</v>
       </c>
       <c r="C105" s="10" t="s">
-        <v>317</v>
+        <v>251</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A106" s="10" t="s">
-        <v>318</v>
+        <v>252</v>
       </c>
       <c r="B106" s="10" t="s">
-        <v>319</v>
+        <v>253</v>
       </c>
       <c r="C106" s="10" t="s">
-        <v>320</v>
+        <v>254</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A107" s="10" t="s">
-        <v>321</v>
+        <v>255</v>
       </c>
       <c r="B107" s="10" t="s">
-        <v>322</v>
+        <v>256</v>
       </c>
       <c r="C107" s="10" t="s">
-        <v>323</v>
+        <v>257</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A108" s="10" t="s">
-        <v>324</v>
+        <v>258</v>
       </c>
       <c r="B108" s="10" t="s">
-        <v>325</v>
+        <v>259</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>326</v>
+        <v>260</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A109" s="10" t="s">
-        <v>327</v>
+        <v>261</v>
       </c>
       <c r="B109" s="10" t="s">
-        <v>328</v>
+        <v>262</v>
       </c>
       <c r="C109" s="10" t="s">
-        <v>329</v>
+        <v>263</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A110" s="10" t="s">
-        <v>330</v>
+        <v>264</v>
       </c>
       <c r="B110" s="10" t="s">
-        <v>331</v>
+        <v>265</v>
       </c>
       <c r="C110" s="10" t="s">
-        <v>332</v>
+        <v>266</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111" s="10" t="s">
-        <v>333</v>
+        <v>267</v>
       </c>
       <c r="B111" s="10" t="s">
-        <v>334</v>
+        <v>268</v>
       </c>
       <c r="C111" s="10" t="s">
-        <v>335</v>
+        <v>269</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112" s="10" t="s">
-        <v>336</v>
+        <v>270</v>
       </c>
       <c r="B112" s="10" t="s">
-        <v>337</v>
+        <v>271</v>
       </c>
       <c r="C112" s="10" t="s">
-        <v>338</v>
+        <v>272</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" s="10" t="s">
-        <v>339</v>
+        <v>273</v>
       </c>
       <c r="B113" s="10" t="s">
-        <v>340</v>
+        <v>274</v>
       </c>
       <c r="C113" s="10" t="s">
-        <v>341</v>
+        <v>275</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" s="10" t="s">
-        <v>342</v>
+        <v>276</v>
       </c>
       <c r="B114" s="10" t="s">
-        <v>343</v>
+        <v>277</v>
       </c>
       <c r="C114" s="10" t="s">
-        <v>344</v>
+        <v>278</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" s="10" t="s">
-        <v>345</v>
+        <v>279</v>
       </c>
       <c r="B115" s="10" t="s">
-        <v>346</v>
+        <v>280</v>
       </c>
       <c r="C115" s="10" t="s">
-        <v>347</v>
+        <v>281</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116" s="10" t="s">
-        <v>348</v>
+        <v>282</v>
       </c>
       <c r="B116" s="10" t="s">
-        <v>349</v>
+        <v>283</v>
       </c>
       <c r="C116" s="10" t="s">
-        <v>350</v>
+        <v>284</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117" s="10" t="s">
-        <v>351</v>
+        <v>285</v>
       </c>
       <c r="B117" s="10" t="s">
-        <v>352</v>
+        <v>286</v>
       </c>
       <c r="C117" s="10" t="s">
-        <v>353</v>
+        <v>287</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118" s="10" t="s">
-        <v>354</v>
+        <v>288</v>
       </c>
       <c r="B118" s="10" t="s">
-        <v>355</v>
+        <v>289</v>
       </c>
       <c r="C118" s="10" t="s">
-        <v>356</v>
+        <v>290</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119" s="10" t="s">
-        <v>357</v>
+        <v>291</v>
       </c>
       <c r="B119" s="10" t="s">
-        <v>358</v>
+        <v>292</v>
       </c>
       <c r="C119" s="10" t="s">
-        <v>359</v>
+        <v>293</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120" s="10" t="s">
-        <v>360</v>
+        <v>294</v>
       </c>
       <c r="B120" s="10" t="s">
-        <v>361</v>
+        <v>295</v>
       </c>
       <c r="C120" s="10" t="s">
-        <v>362</v>
+        <v>296</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A121" s="10" t="s">
-        <v>363</v>
+        <v>297</v>
       </c>
       <c r="B121" s="10" t="s">
-        <v>364</v>
+        <v>298</v>
       </c>
       <c r="C121" s="10" t="s">
-        <v>365</v>
+        <v>299</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A122" s="10" t="s">
-        <v>366</v>
+        <v>300</v>
       </c>
       <c r="B122" s="10" t="s">
-        <v>367</v>
+        <v>301</v>
       </c>
       <c r="C122" s="10" t="s">
-        <v>368</v>
+        <v>302</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" s="10" t="s">
-        <v>369</v>
+        <v>303</v>
       </c>
       <c r="B123" s="10" t="s">
-        <v>370</v>
+        <v>304</v>
       </c>
       <c r="C123" s="10" t="s">
-        <v>371</v>
+        <v>305</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124" s="10" t="s">
-        <v>372</v>
+        <v>306</v>
       </c>
       <c r="B124" s="10" t="s">
-        <v>373</v>
+        <v>307</v>
       </c>
       <c r="C124" s="10" t="s">
-        <v>374</v>
+        <v>308</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125" s="10" t="s">
-        <v>375</v>
+        <v>309</v>
       </c>
       <c r="B125" s="10" t="s">
-        <v>376</v>
+        <v>310</v>
       </c>
       <c r="C125" s="10" t="s">
-        <v>377</v>
+        <v>311</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" s="10" t="s">
-        <v>378</v>
+        <v>312</v>
       </c>
       <c r="B126" s="10" t="s">
-        <v>379</v>
+        <v>313</v>
       </c>
       <c r="C126" s="10" t="s">
-        <v>380</v>
+        <v>314</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A127" s="10" t="s">
-        <v>381</v>
+        <v>315</v>
       </c>
       <c r="B127" s="10" t="s">
-        <v>382</v>
+        <v>316</v>
       </c>
       <c r="C127" s="10" t="s">
-        <v>383</v>
+        <v>317</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128" s="10" t="s">
-        <v>384</v>
+        <v>318</v>
       </c>
       <c r="B128" s="10" t="s">
-        <v>385</v>
+        <v>319</v>
       </c>
       <c r="C128" s="10" t="s">
-        <v>386</v>
+        <v>320</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A129" s="10" t="s">
-        <v>387</v>
+        <v>321</v>
       </c>
       <c r="B129" s="10" t="s">
-        <v>388</v>
+        <v>322</v>
       </c>
       <c r="C129" s="10" t="s">
-        <v>389</v>
+        <v>323</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A130" s="10" t="s">
-        <v>390</v>
+        <v>324</v>
       </c>
       <c r="B130" s="10" t="s">
-        <v>391</v>
+        <v>325</v>
       </c>
       <c r="C130" s="10" t="s">
-        <v>392</v>
+        <v>326</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A131" s="10" t="s">
-        <v>393</v>
+        <v>327</v>
       </c>
       <c r="B131" s="10" t="s">
-        <v>394</v>
+        <v>328</v>
       </c>
       <c r="C131" s="10" t="s">
-        <v>395</v>
+        <v>329</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A132" s="10" t="s">
-        <v>396</v>
+        <v>330</v>
       </c>
       <c r="B132" s="10" t="s">
-        <v>397</v>
+        <v>331</v>
       </c>
       <c r="C132" s="10" t="s">
-        <v>398</v>
+        <v>332</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A133" s="10" t="s">
-        <v>399</v>
+        <v>333</v>
       </c>
       <c r="B133" s="10" t="s">
-        <v>400</v>
+        <v>334</v>
       </c>
       <c r="C133" s="10" t="s">
-        <v>401</v>
+        <v>335</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A134" s="10" t="s">
-        <v>402</v>
+        <v>336</v>
       </c>
       <c r="B134" s="10" t="s">
-        <v>403</v>
+        <v>337</v>
       </c>
       <c r="C134" s="10" t="s">
-        <v>404</v>
+        <v>338</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A135" s="10" t="s">
-        <v>405</v>
+        <v>339</v>
       </c>
       <c r="B135" s="10" t="s">
-        <v>406</v>
+        <v>340</v>
       </c>
       <c r="C135" s="10" t="s">
-        <v>407</v>
+        <v>341</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A136" s="10" t="s">
-        <v>408</v>
+        <v>342</v>
       </c>
       <c r="B136" s="10" t="s">
-        <v>409</v>
+        <v>343</v>
       </c>
       <c r="C136" s="10" t="s">
-        <v>410</v>
+        <v>344</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A137" s="10" t="s">
-        <v>411</v>
+        <v>345</v>
       </c>
       <c r="B137" s="10" t="s">
-        <v>412</v>
+        <v>346</v>
       </c>
       <c r="C137" s="10" t="s">
-        <v>413</v>
+        <v>347</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138" s="10" t="s">
-        <v>414</v>
+        <v>348</v>
       </c>
       <c r="B138" s="10" t="s">
-        <v>415</v>
+        <v>349</v>
       </c>
       <c r="C138" s="10" t="s">
-        <v>416</v>
+        <v>350</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A139" s="10" t="s">
-        <v>417</v>
+        <v>351</v>
       </c>
       <c r="B139" s="10" t="s">
-        <v>418</v>
+        <v>352</v>
       </c>
       <c r="C139" s="10" t="s">
-        <v>419</v>
+        <v>353</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A140" s="10" t="s">
-        <v>420</v>
+        <v>354</v>
       </c>
       <c r="B140" s="10" t="s">
-        <v>421</v>
+        <v>355</v>
       </c>
       <c r="C140" s="10" t="s">
-        <v>422</v>
+        <v>356</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A141" s="10" t="s">
-        <v>423</v>
+        <v>357</v>
       </c>
       <c r="B141" s="10" t="s">
-        <v>424</v>
+        <v>358</v>
       </c>
       <c r="C141" s="10" t="s">
-        <v>425</v>
+        <v>359</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A142" s="10" t="s">
-        <v>426</v>
+        <v>360</v>
       </c>
       <c r="B142" s="10" t="s">
-        <v>427</v>
+        <v>361</v>
       </c>
       <c r="C142" s="10" t="s">
-        <v>428</v>
+        <v>362</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A143" s="10" t="s">
-        <v>429</v>
+        <v>363</v>
       </c>
       <c r="B143" s="10" t="s">
-        <v>430</v>
+        <v>364</v>
       </c>
       <c r="C143" s="10" t="s">
-        <v>431</v>
+        <v>365</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A144" s="10" t="s">
-        <v>432</v>
+        <v>366</v>
       </c>
       <c r="B144" s="10" t="s">
-        <v>433</v>
+        <v>367</v>
       </c>
       <c r="C144" s="10" t="s">
-        <v>434</v>
+        <v>368</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A145" s="10" t="s">
-        <v>435</v>
+        <v>369</v>
       </c>
       <c r="B145" s="10" t="s">
-        <v>436</v>
+        <v>370</v>
       </c>
       <c r="C145" s="10" t="s">
-        <v>437</v>
+        <v>371</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A146" s="10" t="s">
-        <v>438</v>
+        <v>372</v>
       </c>
       <c r="B146" s="10" t="s">
-        <v>439</v>
+        <v>373</v>
       </c>
       <c r="C146" s="10" t="s">
-        <v>440</v>
+        <v>374</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A147" s="10" t="s">
-        <v>441</v>
+        <v>375</v>
       </c>
       <c r="B147" s="10" t="s">
-        <v>442</v>
+        <v>376</v>
       </c>
       <c r="C147" s="10" t="s">
-        <v>443</v>
+        <v>377</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A148" s="10" t="s">
-        <v>444</v>
+        <v>378</v>
       </c>
       <c r="B148" s="10" t="s">
-        <v>445</v>
+        <v>379</v>
       </c>
       <c r="C148" s="10" t="s">
-        <v>446</v>
+        <v>380</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A149" s="10" t="s">
-        <v>447</v>
+        <v>381</v>
       </c>
       <c r="B149" s="10" t="s">
-        <v>448</v>
+        <v>382</v>
       </c>
       <c r="C149" s="10" t="s">
-        <v>449</v>
+        <v>383</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A150" s="10" t="s">
-        <v>450</v>
+        <v>384</v>
       </c>
       <c r="B150" s="10" t="s">
-        <v>451</v>
+        <v>385</v>
       </c>
       <c r="C150" s="10" t="s">
-        <v>452</v>
+        <v>386</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A151" s="10" t="s">
-        <v>453</v>
+        <v>387</v>
       </c>
       <c r="B151" s="10" t="s">
-        <v>454</v>
+        <v>388</v>
       </c>
       <c r="C151" s="10" t="s">
-        <v>455</v>
+        <v>389</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A152" s="10" t="s">
-        <v>456</v>
+        <v>390</v>
       </c>
       <c r="B152" s="10" t="s">
-        <v>457</v>
+        <v>391</v>
       </c>
       <c r="C152" s="10" t="s">
-        <v>458</v>
+        <v>392</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A153" s="10" t="s">
-        <v>459</v>
+        <v>393</v>
       </c>
       <c r="B153" s="10" t="s">
-        <v>460</v>
+        <v>394</v>
       </c>
       <c r="C153" s="10" t="s">
-        <v>461</v>
+        <v>395</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A154" s="10" t="s">
-        <v>462</v>
+        <v>396</v>
       </c>
       <c r="B154" s="10" t="s">
-        <v>463</v>
+        <v>397</v>
       </c>
       <c r="C154" s="10" t="s">
-        <v>464</v>
+        <v>398</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A155" s="10" t="s">
-        <v>465</v>
+        <v>399</v>
       </c>
       <c r="B155" s="10" t="s">
-        <v>466</v>
+        <v>400</v>
       </c>
       <c r="C155" s="10" t="s">
-        <v>467</v>
+        <v>401</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A156" s="10" t="s">
-        <v>468</v>
+        <v>402</v>
       </c>
       <c r="B156" s="10" t="s">
-        <v>469</v>
+        <v>403</v>
       </c>
       <c r="C156" s="10" t="s">
-        <v>470</v>
+        <v>404</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A157" s="10" t="s">
-        <v>471</v>
+        <v>405</v>
       </c>
       <c r="B157" s="10" t="s">
-        <v>472</v>
+        <v>406</v>
       </c>
       <c r="C157" s="10" t="s">
-        <v>473</v>
+        <v>407</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A158" s="10" t="s">
-        <v>474</v>
+        <v>408</v>
       </c>
       <c r="B158" s="10" t="s">
-        <v>475</v>
+        <v>409</v>
       </c>
       <c r="C158" s="10" t="s">
-        <v>476</v>
+        <v>410</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A159" s="10" t="s">
-        <v>477</v>
+        <v>411</v>
       </c>
       <c r="B159" s="10" t="s">
-        <v>478</v>
+        <v>412</v>
       </c>
       <c r="C159" s="10" t="s">
-        <v>479</v>
+        <v>413</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A160" s="10" t="s">
-        <v>480</v>
+        <v>414</v>
       </c>
       <c r="B160" s="10" t="s">
-        <v>481</v>
+        <v>415</v>
       </c>
       <c r="C160" s="10" t="s">
-        <v>482</v>
+        <v>416</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A161" s="10" t="s">
-        <v>483</v>
+        <v>417</v>
       </c>
       <c r="B161" s="10" t="s">
-        <v>484</v>
+        <v>418</v>
       </c>
       <c r="C161" s="10" t="s">
-        <v>485</v>
+        <v>419</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A162" s="10" t="s">
-        <v>486</v>
+        <v>420</v>
       </c>
       <c r="B162" s="10" t="s">
-        <v>487</v>
+        <v>421</v>
       </c>
       <c r="C162" s="10" t="s">
-        <v>488</v>
+        <v>422</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A163" s="10" t="s">
-        <v>489</v>
+        <v>423</v>
       </c>
       <c r="B163" s="10" t="s">
-        <v>490</v>
+        <v>424</v>
       </c>
       <c r="C163" s="10" t="s">
-        <v>491</v>
+        <v>425</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A164" s="10" t="s">
-        <v>492</v>
+        <v>426</v>
       </c>
       <c r="B164" s="10" t="s">
-        <v>493</v>
+        <v>427</v>
       </c>
       <c r="C164" s="10" t="s">
-        <v>494</v>
+        <v>428</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A165" s="10" t="s">
-        <v>495</v>
+        <v>429</v>
       </c>
       <c r="B165" s="10" t="s">
-        <v>496</v>
+        <v>430</v>
       </c>
       <c r="C165" s="10" t="s">
-        <v>497</v>
+        <v>431</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A166" s="10" t="s">
-        <v>498</v>
+        <v>432</v>
       </c>
       <c r="B166" s="10" t="s">
-        <v>499</v>
+        <v>433</v>
       </c>
       <c r="C166" s="10" t="s">
-        <v>500</v>
+        <v>434</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A167" s="10" t="s">
-        <v>501</v>
+        <v>435</v>
       </c>
       <c r="B167" s="10" t="s">
-        <v>502</v>
+        <v>436</v>
       </c>
       <c r="C167" s="10" t="s">
-        <v>503</v>
+        <v>437</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A168" s="10" t="s">
-        <v>504</v>
+        <v>438</v>
       </c>
       <c r="B168" s="10" t="s">
-        <v>505</v>
+        <v>439</v>
       </c>
       <c r="C168" s="10" t="s">
-        <v>506</v>
+        <v>440</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A169" s="10" t="s">
-        <v>507</v>
+        <v>441</v>
       </c>
       <c r="B169" s="10" t="s">
-        <v>508</v>
+        <v>442</v>
       </c>
       <c r="C169" s="10" t="s">
-        <v>509</v>
+        <v>443</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A170" s="10" t="s">
-        <v>510</v>
+        <v>444</v>
       </c>
       <c r="B170" s="10" t="s">
-        <v>511</v>
+        <v>445</v>
       </c>
       <c r="C170" s="10" t="s">
-        <v>512</v>
+        <v>446</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A171" s="10" t="s">
-        <v>513</v>
+        <v>447</v>
       </c>
       <c r="B171" s="10" t="s">
-        <v>514</v>
+        <v>448</v>
       </c>
       <c r="C171" s="10" t="s">
-        <v>515</v>
+        <v>449</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A172" s="10" t="s">
-        <v>516</v>
+        <v>450</v>
       </c>
       <c r="B172" s="10" t="s">
-        <v>517</v>
+        <v>451</v>
       </c>
       <c r="C172" s="10" t="s">
-        <v>518</v>
+        <v>452</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A173" s="10" t="s">
-        <v>519</v>
+        <v>453</v>
       </c>
       <c r="B173" s="10" t="s">
-        <v>520</v>
+        <v>454</v>
       </c>
       <c r="C173" s="10" t="s">
-        <v>521</v>
+        <v>455</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A174" s="10" t="s">
-        <v>522</v>
+        <v>456</v>
       </c>
       <c r="B174" s="10" t="s">
-        <v>523</v>
+        <v>457</v>
       </c>
       <c r="C174" s="10" t="s">
-        <v>524</v>
+        <v>458</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A175" s="10" t="s">
-        <v>525</v>
+        <v>459</v>
       </c>
       <c r="B175" s="10" t="s">
-        <v>526</v>
+        <v>460</v>
       </c>
       <c r="C175" s="10" t="s">
-        <v>527</v>
+        <v>461</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A176" s="10" t="s">
-        <v>528</v>
+        <v>462</v>
       </c>
       <c r="B176" s="10" t="s">
-        <v>529</v>
+        <v>463</v>
       </c>
       <c r="C176" s="10" t="s">
-        <v>530</v>
+        <v>464</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A177" s="10" t="s">
-        <v>531</v>
+        <v>465</v>
       </c>
       <c r="B177" s="10" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="C177" s="10" t="s">
-        <v>533</v>
+        <v>467</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A178" s="10" t="s">
-        <v>534</v>
+        <v>468</v>
       </c>
       <c r="B178" s="10" t="s">
-        <v>535</v>
+        <v>469</v>
       </c>
       <c r="C178" s="10" t="s">
-        <v>536</v>
+        <v>470</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A179" s="10" t="s">
-        <v>537</v>
+        <v>471</v>
       </c>
       <c r="B179" s="10" t="s">
-        <v>538</v>
+        <v>472</v>
       </c>
       <c r="C179" s="10" t="s">
-        <v>539</v>
+        <v>473</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A180" s="10" t="s">
-        <v>540</v>
+        <v>474</v>
       </c>
       <c r="B180" s="10" t="s">
-        <v>541</v>
+        <v>475</v>
       </c>
       <c r="C180" s="10" t="s">
-        <v>542</v>
+        <v>476</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A181" s="10" t="s">
-        <v>543</v>
+        <v>477</v>
       </c>
       <c r="B181" s="10" t="s">
-        <v>544</v>
+        <v>478</v>
       </c>
       <c r="C181" s="10" t="s">
-        <v>545</v>
+        <v>479</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A182" s="10" t="s">
-        <v>546</v>
+        <v>480</v>
       </c>
       <c r="B182" s="10" t="s">
-        <v>547</v>
+        <v>481</v>
       </c>
       <c r="C182" s="10" t="s">
-        <v>548</v>
+        <v>482</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A183" s="10" t="s">
-        <v>549</v>
+        <v>483</v>
       </c>
       <c r="B183" s="10" t="s">
-        <v>550</v>
+        <v>484</v>
       </c>
       <c r="C183" s="10" t="s">
-        <v>551</v>
+        <v>485</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A184" s="10" t="s">
-        <v>552</v>
+        <v>486</v>
       </c>
       <c r="B184" s="10" t="s">
-        <v>553</v>
+        <v>487</v>
       </c>
       <c r="C184" s="10" t="s">
-        <v>554</v>
+        <v>488</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A185" s="10" t="s">
-        <v>555</v>
+        <v>489</v>
       </c>
       <c r="B185" s="10" t="s">
-        <v>556</v>
+        <v>490</v>
       </c>
       <c r="C185" s="10" t="s">
-        <v>557</v>
+        <v>491</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A186" s="10" t="s">
-        <v>558</v>
+        <v>492</v>
       </c>
       <c r="B186" s="10" t="s">
-        <v>559</v>
+        <v>493</v>
       </c>
       <c r="C186" s="10" t="s">
-        <v>560</v>
+        <v>494</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A187" s="10" t="s">
-        <v>561</v>
+        <v>495</v>
       </c>
       <c r="B187" s="10" t="s">
-        <v>562</v>
+        <v>496</v>
       </c>
       <c r="C187" s="10" t="s">
-        <v>563</v>
+        <v>497</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A188" s="10" t="s">
-        <v>564</v>
+        <v>498</v>
       </c>
       <c r="B188" s="10" t="s">
-        <v>565</v>
+        <v>499</v>
       </c>
       <c r="C188" s="10" t="s">
-        <v>566</v>
+        <v>500</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A189" s="10" t="s">
-        <v>567</v>
+        <v>501</v>
       </c>
       <c r="B189" s="10" t="s">
-        <v>568</v>
+        <v>502</v>
       </c>
       <c r="C189" s="10" t="s">
-        <v>569</v>
+        <v>503</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A190" s="10" t="s">
-        <v>570</v>
+        <v>504</v>
       </c>
       <c r="B190" s="10" t="s">
-        <v>571</v>
+        <v>505</v>
       </c>
       <c r="C190" s="10" t="s">
-        <v>572</v>
+        <v>506</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A191" s="10" t="s">
-        <v>573</v>
+        <v>507</v>
       </c>
       <c r="B191" s="10" t="s">
-        <v>574</v>
+        <v>508</v>
       </c>
       <c r="C191" s="10" t="s">
-        <v>575</v>
+        <v>509</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A192" s="10" t="s">
-        <v>576</v>
+        <v>510</v>
       </c>
       <c r="B192" s="10" t="s">
-        <v>577</v>
+        <v>511</v>
       </c>
       <c r="C192" s="10" t="s">
-        <v>578</v>
+        <v>512</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A193" s="10" t="s">
-        <v>579</v>
+        <v>513</v>
       </c>
       <c r="B193" s="10" t="s">
-        <v>580</v>
+        <v>514</v>
       </c>
       <c r="C193" s="10" t="s">
-        <v>581</v>
+        <v>515</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A194" s="10" t="s">
-        <v>582</v>
+        <v>516</v>
       </c>
       <c r="B194" s="10" t="s">
-        <v>583</v>
+        <v>517</v>
       </c>
       <c r="C194" s="10" t="s">
-        <v>584</v>
+        <v>518</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A195" s="10" t="s">
-        <v>585</v>
+        <v>519</v>
       </c>
       <c r="B195" s="10" t="s">
-        <v>586</v>
+        <v>520</v>
       </c>
       <c r="C195" s="10" t="s">
-        <v>587</v>
+        <v>521</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A196" s="10" t="s">
-        <v>588</v>
+        <v>522</v>
       </c>
       <c r="B196" s="10" t="s">
-        <v>589</v>
+        <v>523</v>
       </c>
       <c r="C196" s="10" t="s">
-        <v>590</v>
+        <v>524</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A197" s="10" t="s">
-        <v>591</v>
+        <v>525</v>
       </c>
       <c r="B197" s="10" t="s">
-        <v>592</v>
+        <v>526</v>
       </c>
       <c r="C197" s="10" t="s">
-        <v>593</v>
+        <v>527</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A198" s="10" t="s">
-        <v>594</v>
+        <v>528</v>
       </c>
       <c r="B198" s="10" t="s">
-        <v>595</v>
+        <v>529</v>
       </c>
       <c r="C198" s="10" t="s">
-        <v>596</v>
+        <v>530</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A199" s="10" t="s">
-        <v>597</v>
+        <v>531</v>
       </c>
       <c r="B199" s="10" t="s">
-        <v>598</v>
+        <v>532</v>
       </c>
       <c r="C199" s="10" t="s">
-        <v>599</v>
+        <v>533</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A200" s="10" t="s">
-        <v>600</v>
+        <v>534</v>
       </c>
       <c r="B200" s="10" t="s">
-        <v>601</v>
+        <v>535</v>
       </c>
       <c r="C200" s="10" t="s">
-        <v>602</v>
+        <v>536</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A201" s="10" t="s">
-        <v>603</v>
+        <v>537</v>
       </c>
       <c r="B201" s="10" t="s">
-        <v>604</v>
+        <v>538</v>
       </c>
       <c r="C201" s="10" t="s">
-        <v>605</v>
+        <v>539</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A202" s="10" t="s">
-        <v>606</v>
+        <v>540</v>
       </c>
       <c r="B202" s="10" t="s">
-        <v>607</v>
+        <v>541</v>
       </c>
       <c r="C202" s="10" t="s">
-        <v>608</v>
+        <v>542</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A203" s="10" t="s">
-        <v>609</v>
+        <v>543</v>
       </c>
       <c r="B203" s="10" t="s">
-        <v>610</v>
+        <v>544</v>
       </c>
       <c r="C203" s="10" t="s">
-        <v>611</v>
+        <v>545</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A204" s="10" t="s">
-        <v>612</v>
+        <v>546</v>
       </c>
       <c r="B204" s="10" t="s">
-        <v>613</v>
+        <v>547</v>
       </c>
       <c r="C204" s="10" t="s">
-        <v>614</v>
+        <v>548</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A205" s="10" t="s">
-        <v>615</v>
+        <v>549</v>
       </c>
       <c r="B205" s="10" t="s">
-        <v>616</v>
+        <v>550</v>
       </c>
       <c r="C205" s="10" t="s">
-        <v>617</v>
+        <v>551</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A206" s="10" t="s">
-        <v>618</v>
+        <v>552</v>
       </c>
       <c r="B206" s="10" t="s">
-        <v>619</v>
+        <v>553</v>
       </c>
       <c r="C206" s="10" t="s">
-        <v>620</v>
+        <v>554</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A207" s="10" t="s">
-        <v>621</v>
+        <v>555</v>
       </c>
       <c r="B207" s="10" t="s">
-        <v>622</v>
+        <v>556</v>
       </c>
       <c r="C207" s="10" t="s">
-        <v>623</v>
+        <v>557</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A208" s="10" t="s">
-        <v>624</v>
+        <v>558</v>
       </c>
       <c r="B208" s="10" t="s">
-        <v>625</v>
+        <v>559</v>
       </c>
       <c r="C208" s="10" t="s">
-        <v>626</v>
+        <v>560</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A209" s="10" t="s">
-        <v>627</v>
+        <v>561</v>
       </c>
       <c r="B209" s="10" t="s">
-        <v>628</v>
+        <v>562</v>
       </c>
       <c r="C209" s="10" t="s">
-        <v>629</v>
+        <v>563</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A210" s="10" t="s">
-        <v>630</v>
+        <v>564</v>
       </c>
       <c r="B210" s="10" t="s">
-        <v>631</v>
+        <v>565</v>
       </c>
       <c r="C210" s="10" t="s">
-        <v>632</v>
+        <v>566</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A211" s="10" t="s">
-        <v>633</v>
+        <v>567</v>
       </c>
       <c r="B211" s="10" t="s">
-        <v>634</v>
+        <v>568</v>
       </c>
       <c r="C211" s="10" t="s">
-        <v>635</v>
+        <v>569</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A212" s="10" t="s">
-        <v>636</v>
+        <v>570</v>
       </c>
       <c r="B212" s="10" t="s">
-        <v>637</v>
+        <v>571</v>
       </c>
       <c r="C212" s="10" t="s">
-        <v>638</v>
+        <v>572</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A213" s="10" t="s">
-        <v>639</v>
+        <v>573</v>
       </c>
       <c r="B213" s="10" t="s">
-        <v>640</v>
+        <v>574</v>
       </c>
       <c r="C213" s="10" t="s">
-        <v>641</v>
+        <v>575</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A214" s="10" t="s">
-        <v>642</v>
+        <v>576</v>
       </c>
       <c r="B214" s="10" t="s">
-        <v>643</v>
+        <v>577</v>
       </c>
       <c r="C214" s="10" t="s">
-        <v>644</v>
+        <v>578</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A215" s="10" t="s">
-        <v>645</v>
+        <v>579</v>
       </c>
       <c r="B215" s="10" t="s">
-        <v>646</v>
+        <v>580</v>
       </c>
       <c r="C215" s="10" t="s">
-        <v>647</v>
+        <v>581</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A216" s="10" t="s">
-        <v>648</v>
+        <v>582</v>
       </c>
       <c r="B216" s="10" t="s">
-        <v>649</v>
+        <v>583</v>
       </c>
       <c r="C216" s="10" t="s">
-        <v>650</v>
+        <v>584</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A217" s="10" t="s">
-        <v>651</v>
+        <v>585</v>
       </c>
       <c r="B217" s="10" t="s">
-        <v>652</v>
+        <v>586</v>
       </c>
       <c r="C217" s="10" t="s">
-        <v>653</v>
+        <v>587</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A218" s="10" t="s">
-        <v>654</v>
+        <v>588</v>
       </c>
       <c r="B218" s="10" t="s">
-        <v>655</v>
+        <v>589</v>
       </c>
       <c r="C218" s="10" t="s">
-        <v>656</v>
+        <v>590</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A219" s="10" t="s">
-        <v>657</v>
+        <v>591</v>
       </c>
       <c r="B219" s="10" t="s">
-        <v>658</v>
+        <v>592</v>
       </c>
       <c r="C219" s="10" t="s">
-        <v>659</v>
+        <v>593</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A220" s="10" t="s">
-        <v>660</v>
+        <v>594</v>
       </c>
       <c r="B220" s="10" t="s">
-        <v>661</v>
+        <v>595</v>
       </c>
       <c r="C220" s="10" t="s">
-        <v>662</v>
+        <v>596</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A221" s="10" t="s">
-        <v>663</v>
+        <v>597</v>
       </c>
       <c r="B221" s="10" t="s">
-        <v>664</v>
+        <v>598</v>
       </c>
       <c r="C221" s="10" t="s">
-        <v>665</v>
+        <v>599</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A222" s="10" t="s">
-        <v>666</v>
+        <v>600</v>
       </c>
       <c r="B222" s="10" t="s">
-        <v>667</v>
+        <v>601</v>
       </c>
       <c r="C222" s="10" t="s">
-        <v>668</v>
+        <v>602</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A223" s="10" t="s">
-        <v>669</v>
+        <v>603</v>
       </c>
       <c r="B223" s="10" t="s">
-        <v>670</v>
+        <v>604</v>
       </c>
       <c r="C223" s="10" t="s">
-        <v>671</v>
+        <v>605</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A224" s="10" t="s">
-        <v>672</v>
+        <v>606</v>
       </c>
       <c r="B224" s="10" t="s">
-        <v>673</v>
+        <v>607</v>
       </c>
       <c r="C224" s="10" t="s">
-        <v>674</v>
+        <v>608</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A225" s="10" t="s">
-        <v>675</v>
+        <v>609</v>
       </c>
       <c r="B225" s="10" t="s">
-        <v>676</v>
+        <v>610</v>
       </c>
       <c r="C225" s="10" t="s">
-        <v>677</v>
+        <v>611</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A226" s="10" t="s">
-        <v>678</v>
+        <v>612</v>
       </c>
       <c r="B226" s="10" t="s">
-        <v>679</v>
+        <v>613</v>
       </c>
       <c r="C226" s="10" t="s">
-        <v>680</v>
+        <v>614</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A227" s="10" t="s">
-        <v>681</v>
+        <v>615</v>
       </c>
       <c r="B227" s="10" t="s">
-        <v>682</v>
+        <v>616</v>
       </c>
       <c r="C227" s="10" t="s">
-        <v>683</v>
+        <v>617</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A228" s="10" t="s">
-        <v>684</v>
+        <v>618</v>
       </c>
       <c r="B228" s="10" t="s">
-        <v>685</v>
+        <v>619</v>
       </c>
       <c r="C228" s="10" t="s">
-        <v>686</v>
+        <v>620</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A229" s="10" t="s">
-        <v>687</v>
+        <v>621</v>
       </c>
       <c r="B229" s="10" t="s">
-        <v>688</v>
+        <v>622</v>
       </c>
       <c r="C229" s="10" t="s">
-        <v>689</v>
+        <v>623</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A230" s="10" t="s">
-        <v>690</v>
+        <v>624</v>
       </c>
       <c r="B230" s="10" t="s">
-        <v>691</v>
+        <v>625</v>
       </c>
       <c r="C230" s="10" t="s">
-        <v>692</v>
+        <v>626</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A231" s="10" t="s">
-        <v>693</v>
+        <v>627</v>
       </c>
       <c r="B231" s="10" t="s">
-        <v>694</v>
+        <v>628</v>
       </c>
       <c r="C231" s="10" t="s">
-        <v>695</v>
+        <v>629</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A232" s="10" t="s">
-        <v>696</v>
+        <v>630</v>
       </c>
       <c r="B232" s="10" t="s">
-        <v>697</v>
+        <v>631</v>
       </c>
       <c r="C232" s="10" t="s">
-        <v>698</v>
+        <v>632</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A233" s="10" t="s">
-        <v>699</v>
+        <v>633</v>
       </c>
       <c r="B233" s="10" t="s">
-        <v>700</v>
+        <v>634</v>
       </c>
       <c r="C233" s="10" t="s">
-        <v>701</v>
+        <v>635</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A234" s="10" t="s">
-        <v>702</v>
+        <v>636</v>
       </c>
       <c r="B234" s="10" t="s">
-        <v>703</v>
+        <v>637</v>
       </c>
       <c r="C234" s="10" t="s">
-        <v>704</v>
+        <v>638</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A235" s="10" t="s">
-        <v>705</v>
+        <v>639</v>
       </c>
       <c r="B235" s="10" t="s">
-        <v>706</v>
+        <v>640</v>
       </c>
       <c r="C235" s="10" t="s">
-        <v>707</v>
+        <v>641</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A236" s="10" t="s">
-        <v>708</v>
+        <v>642</v>
       </c>
       <c r="B236" s="10" t="s">
-        <v>709</v>
+        <v>643</v>
       </c>
       <c r="C236" s="10" t="s">
-        <v>710</v>
+        <v>644</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A237" s="10" t="s">
-        <v>711</v>
+        <v>645</v>
       </c>
       <c r="B237" s="10" t="s">
-        <v>712</v>
+        <v>646</v>
       </c>
       <c r="C237" s="10" t="s">
-        <v>713</v>
+        <v>647</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A238" s="10" t="s">
-        <v>714</v>
+        <v>648</v>
       </c>
       <c r="B238" s="10" t="s">
-        <v>715</v>
+        <v>649</v>
       </c>
       <c r="C238" s="10" t="s">
-        <v>716</v>
+        <v>650</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A239" s="10" t="s">
-        <v>717</v>
+        <v>651</v>
       </c>
       <c r="B239" s="10" t="s">
-        <v>718</v>
+        <v>652</v>
       </c>
       <c r="C239" s="10" t="s">
-        <v>719</v>
+        <v>653</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A240" s="10" t="s">
-        <v>720</v>
+        <v>654</v>
       </c>
       <c r="B240" s="10" t="s">
-        <v>721</v>
+        <v>655</v>
       </c>
       <c r="C240" s="10" t="s">
-        <v>722</v>
+        <v>656</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A241" s="10" t="s">
-        <v>723</v>
+        <v>657</v>
       </c>
       <c r="B241" s="10" t="s">
-        <v>724</v>
+        <v>658</v>
       </c>
       <c r="C241" s="10" t="s">
-        <v>725</v>
+        <v>659</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A242" s="10" t="s">
-        <v>726</v>
+        <v>660</v>
       </c>
       <c r="B242" s="10" t="s">
-        <v>727</v>
+        <v>661</v>
       </c>
       <c r="C242" s="10" t="s">
-        <v>728</v>
+        <v>662</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A243" s="10" t="s">
-        <v>729</v>
+        <v>663</v>
       </c>
       <c r="B243" s="10" t="s">
-        <v>730</v>
+        <v>664</v>
       </c>
       <c r="C243" s="10" t="s">
-        <v>731</v>
+        <v>665</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A244" s="10" t="s">
-        <v>732</v>
+        <v>666</v>
       </c>
       <c r="B244" s="10" t="s">
-        <v>733</v>
+        <v>667</v>
       </c>
       <c r="C244" s="10" t="s">
-        <v>734</v>
+        <v>668</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A245" s="10" t="s">
-        <v>735</v>
+        <v>669</v>
       </c>
       <c r="B245" s="10" t="s">
-        <v>736</v>
+        <v>670</v>
       </c>
       <c r="C245" s="10" t="s">
-        <v>737</v>
+        <v>671</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A246" s="10" t="s">
-        <v>738</v>
+        <v>672</v>
       </c>
       <c r="B246" s="10" t="s">
-        <v>739</v>
+        <v>673</v>
       </c>
       <c r="C246" s="10" t="s">
-        <v>740</v>
+        <v>674</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A247" s="10" t="s">
-        <v>741</v>
+        <v>675</v>
       </c>
       <c r="B247" s="10" t="s">
-        <v>742</v>
+        <v>676</v>
       </c>
       <c r="C247" s="10" t="s">
-        <v>743</v>
+        <v>677</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A248" s="10" t="s">
-        <v>744</v>
+        <v>678</v>
       </c>
       <c r="B248" s="10" t="s">
-        <v>745</v>
+        <v>679</v>
       </c>
       <c r="C248" s="10" t="s">
-        <v>746</v>
+        <v>680</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A249" s="10" t="s">
-        <v>747</v>
+        <v>681</v>
       </c>
       <c r="B249" s="10" t="s">
-        <v>748</v>
+        <v>682</v>
       </c>
       <c r="C249" s="10" t="s">
-        <v>749</v>
+        <v>683</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A250" s="10" t="s">
-        <v>750</v>
+        <v>684</v>
       </c>
       <c r="B250" s="10" t="s">
-        <v>751</v>
+        <v>685</v>
       </c>
       <c r="C250" s="10" t="s">
-        <v>752</v>
+        <v>686</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A251" s="10" t="s">
-        <v>753</v>
+        <v>687</v>
       </c>
       <c r="B251" s="10" t="s">
-        <v>754</v>
+        <v>688</v>
       </c>
       <c r="C251" s="10" t="s">
-        <v>755</v>
+        <v>689</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A252" s="10" t="s">
-        <v>756</v>
+        <v>690</v>
       </c>
       <c r="B252" s="10" t="s">
-        <v>757</v>
+        <v>691</v>
       </c>
       <c r="C252" s="10" t="s">
-        <v>758</v>
+        <v>692</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A253" s="10" t="s">
-        <v>759</v>
+        <v>693</v>
       </c>
       <c r="B253" s="10" t="s">
-        <v>760</v>
+        <v>694</v>
       </c>
       <c r="C253" s="10" t="s">
-        <v>761</v>
+        <v>695</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A254" s="10" t="s">
-        <v>762</v>
+        <v>696</v>
       </c>
       <c r="B254" s="10" t="s">
-        <v>763</v>
+        <v>697</v>
       </c>
       <c r="C254" s="10" t="s">
-        <v>764</v>
+        <v>698</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A255" s="10" t="s">
-        <v>765</v>
+        <v>699</v>
       </c>
       <c r="B255" s="10" t="s">
-        <v>766</v>
+        <v>700</v>
       </c>
       <c r="C255" s="10" t="s">
-        <v>767</v>
+        <v>701</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A256" s="10" t="s">
-        <v>768</v>
+        <v>702</v>
       </c>
       <c r="B256" s="10" t="s">
-        <v>769</v>
+        <v>703</v>
       </c>
       <c r="C256" s="10" t="s">
-        <v>770</v>
+        <v>704</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A257" s="10" t="s">
-        <v>771</v>
+        <v>705</v>
       </c>
       <c r="B257" s="10" t="s">
-        <v>772</v>
+        <v>706</v>
       </c>
       <c r="C257" s="10" t="s">
-        <v>773</v>
+        <v>707</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A258" s="10" t="s">
-        <v>774</v>
+        <v>708</v>
       </c>
       <c r="B258" s="10" t="s">
-        <v>775</v>
+        <v>709</v>
       </c>
       <c r="C258" s="10" t="s">
-        <v>776</v>
+        <v>710</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A259" s="10" t="s">
-        <v>777</v>
+        <v>711</v>
       </c>
       <c r="B259" s="10" t="s">
-        <v>778</v>
+        <v>712</v>
       </c>
       <c r="C259" s="10" t="s">
-        <v>779</v>
+        <v>713</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A260" s="10" t="s">
-        <v>780</v>
+        <v>714</v>
       </c>
       <c r="B260" s="10" t="s">
-        <v>781</v>
+        <v>715</v>
       </c>
       <c r="C260" s="10" t="s">
-        <v>782</v>
+        <v>716</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A261" s="10" t="s">
-        <v>783</v>
+        <v>717</v>
       </c>
       <c r="B261" s="10" t="s">
-        <v>784</v>
+        <v>718</v>
       </c>
       <c r="C261" s="10" t="s">
-        <v>785</v>
+        <v>719</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A262" s="10" t="s">
-        <v>786</v>
+        <v>720</v>
       </c>
       <c r="B262" s="10" t="s">
-        <v>787</v>
+        <v>721</v>
       </c>
       <c r="C262" s="10" t="s">
-        <v>788</v>
+        <v>722</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A263" s="10" t="s">
-        <v>789</v>
+        <v>723</v>
       </c>
       <c r="B263" s="10" t="s">
-        <v>790</v>
+        <v>724</v>
       </c>
       <c r="C263" s="10" t="s">
-        <v>791</v>
+        <v>725</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A264" s="10" t="s">
-        <v>792</v>
+        <v>726</v>
       </c>
       <c r="B264" s="10" t="s">
-        <v>793</v>
+        <v>727</v>
       </c>
       <c r="C264" s="10" t="s">
-        <v>794</v>
+        <v>728</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A265" s="10" t="s">
-        <v>795</v>
+        <v>729</v>
       </c>
       <c r="B265" s="10" t="s">
-        <v>796</v>
+        <v>730</v>
       </c>
       <c r="C265" s="10" t="s">
-        <v>797</v>
+        <v>731</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A266" s="10" t="s">
-        <v>798</v>
+        <v>732</v>
       </c>
       <c r="B266" s="10" t="s">
-        <v>799</v>
+        <v>733</v>
       </c>
       <c r="C266" s="10" t="s">
-        <v>800</v>
+        <v>734</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A267" s="10" t="s">
-        <v>801</v>
+        <v>735</v>
       </c>
       <c r="B267" s="10" t="s">
-        <v>802</v>
+        <v>736</v>
       </c>
       <c r="C267" s="10" t="s">
-        <v>803</v>
+        <v>737</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A268" s="10" t="s">
-        <v>804</v>
+        <v>738</v>
       </c>
       <c r="B268" s="10" t="s">
-        <v>805</v>
+        <v>739</v>
       </c>
       <c r="C268" s="10" t="s">
-        <v>806</v>
+        <v>740</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A269" s="10" t="s">
-        <v>807</v>
+        <v>741</v>
       </c>
       <c r="B269" s="10" t="s">
-        <v>808</v>
+        <v>742</v>
       </c>
       <c r="C269" s="10" t="s">
-        <v>809</v>
+        <v>743</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A270" s="10" t="s">
-        <v>810</v>
+        <v>744</v>
       </c>
       <c r="B270" s="10" t="s">
-        <v>811</v>
+        <v>745</v>
       </c>
       <c r="C270" s="10" t="s">
-        <v>812</v>
+        <v>746</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A271" s="10" t="s">
-        <v>813</v>
+        <v>747</v>
       </c>
       <c r="B271" s="10" t="s">
-        <v>814</v>
+        <v>748</v>
       </c>
       <c r="C271" s="10" t="s">
-        <v>815</v>
+        <v>749</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A272" s="10" t="s">
-        <v>816</v>
+        <v>750</v>
       </c>
       <c r="B272" s="10" t="s">
-        <v>817</v>
+        <v>751</v>
       </c>
       <c r="C272" s="10" t="s">
-        <v>818</v>
+        <v>752</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A273" s="10" t="s">
-        <v>819</v>
+        <v>753</v>
       </c>
       <c r="B273" s="10" t="s">
-        <v>820</v>
+        <v>754</v>
       </c>
       <c r="C273" s="10" t="s">
-        <v>821</v>
+        <v>755</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A274" s="10" t="s">
-        <v>822</v>
+        <v>756</v>
       </c>
       <c r="B274" s="10" t="s">
-        <v>823</v>
+        <v>757</v>
       </c>
       <c r="C274" s="10" t="s">
-        <v>824</v>
+        <v>758</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A275" s="10" t="s">
-        <v>825</v>
+        <v>759</v>
       </c>
       <c r="B275" s="10" t="s">
-        <v>826</v>
+        <v>760</v>
       </c>
       <c r="C275" s="10" t="s">
-        <v>827</v>
+        <v>761</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A276" s="10" t="s">
-        <v>828</v>
+        <v>762</v>
       </c>
       <c r="B276" s="10" t="s">
-        <v>829</v>
+        <v>763</v>
       </c>
       <c r="C276" s="10" t="s">
-        <v>830</v>
+        <v>764</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A277" s="10" t="s">
-        <v>831</v>
+        <v>765</v>
       </c>
       <c r="B277" s="10" t="s">
-        <v>832</v>
+        <v>766</v>
       </c>
       <c r="C277" s="10" t="s">
-        <v>833</v>
+        <v>767</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A278" s="10" t="s">
-        <v>834</v>
+        <v>768</v>
       </c>
       <c r="B278" s="10" t="s">
-        <v>835</v>
+        <v>769</v>
       </c>
       <c r="C278" s="10" t="s">
-        <v>836</v>
+        <v>770</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A279" s="10" t="s">
-        <v>837</v>
+        <v>771</v>
       </c>
       <c r="B279" s="10" t="s">
-        <v>838</v>
+        <v>772</v>
       </c>
       <c r="C279" s="10" t="s">
-        <v>839</v>
+        <v>773</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A280" s="10" t="s">
-        <v>840</v>
+        <v>774</v>
       </c>
       <c r="B280" s="10" t="s">
-        <v>841</v>
+        <v>775</v>
       </c>
       <c r="C280" s="10" t="s">
-        <v>842</v>
+        <v>776</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A281" s="10" t="s">
-        <v>843</v>
+        <v>777</v>
       </c>
       <c r="B281" s="10" t="s">
-        <v>844</v>
+        <v>778</v>
       </c>
       <c r="C281" s="10" t="s">
-        <v>845</v>
+        <v>779</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A282" s="10" t="s">
-        <v>846</v>
+        <v>780</v>
       </c>
       <c r="B282" s="10" t="s">
-        <v>847</v>
+        <v>781</v>
       </c>
       <c r="C282" s="10" t="s">
-        <v>848</v>
+        <v>782</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A283" s="10" t="s">
-        <v>849</v>
+        <v>783</v>
       </c>
       <c r="B283" s="10" t="s">
-        <v>850</v>
+        <v>784</v>
       </c>
       <c r="C283" s="10" t="s">
-        <v>851</v>
+        <v>785</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A284" s="10" t="s">
-        <v>852</v>
+        <v>786</v>
       </c>
       <c r="B284" s="10" t="s">
-        <v>853</v>
+        <v>787</v>
       </c>
       <c r="C284" s="10" t="s">
-        <v>854</v>
+        <v>788</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A285" s="10" t="s">
-        <v>855</v>
+        <v>789</v>
       </c>
       <c r="B285" s="10" t="s">
-        <v>856</v>
+        <v>790</v>
       </c>
       <c r="C285" s="10" t="s">
-        <v>857</v>
+        <v>791</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A286" s="10" t="s">
-        <v>858</v>
+        <v>792</v>
       </c>
       <c r="B286" s="10" t="s">
-        <v>859</v>
+        <v>793</v>
       </c>
       <c r="C286" s="10" t="s">
-        <v>860</v>
+        <v>794</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A287" s="10" t="s">
-        <v>861</v>
+        <v>795</v>
       </c>
       <c r="B287" s="10" t="s">
-        <v>862</v>
+        <v>796</v>
       </c>
       <c r="C287" s="10" t="s">
-        <v>863</v>
+        <v>797</v>
       </c>
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A288" s="10" t="s">
-        <v>864</v>
+        <v>798</v>
       </c>
       <c r="B288" s="10" t="s">
-        <v>865</v>
+        <v>799</v>
       </c>
       <c r="C288" s="10" t="s">
-        <v>866</v>
+        <v>800</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A289" s="10" t="s">
-        <v>867</v>
+        <v>801</v>
       </c>
       <c r="B289" s="10" t="s">
-        <v>868</v>
+        <v>802</v>
       </c>
       <c r="C289" s="10" t="s">
-        <v>869</v>
+        <v>803</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A290" s="10" t="s">
-        <v>870</v>
+        <v>804</v>
       </c>
       <c r="B290" s="10" t="s">
-        <v>871</v>
+        <v>805</v>
       </c>
       <c r="C290" s="10" t="s">
-        <v>872</v>
+        <v>806</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A291" s="10" t="s">
-        <v>873</v>
+        <v>807</v>
       </c>
       <c r="B291" s="10" t="s">
-        <v>874</v>
+        <v>808</v>
       </c>
       <c r="C291" s="10" t="s">
-        <v>875</v>
+        <v>809</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A292" s="10" t="s">
-        <v>876</v>
+        <v>810</v>
       </c>
       <c r="B292" s="10" t="s">
-        <v>877</v>
+        <v>811</v>
       </c>
       <c r="C292" s="10" t="s">
-        <v>878</v>
+        <v>812</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A293" s="10" t="s">
+        <v>813</v>
+      </c>
+      <c r="B293" s="10" t="s">
+        <v>814</v>
+      </c>
+      <c r="C293" s="10" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="294" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A294" s="10" t="s">
+        <v>816</v>
+      </c>
+      <c r="B294" s="10" t="s">
+        <v>817</v>
+      </c>
+      <c r="C294" s="10" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="295" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A295" s="10" t="s">
+        <v>819</v>
+      </c>
+      <c r="B295" s="10" t="s">
+        <v>820</v>
+      </c>
+      <c r="C295" s="10" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A296" s="10" t="s">
+        <v>822</v>
+      </c>
+      <c r="B296" s="10" t="s">
+        <v>823</v>
+      </c>
+      <c r="C296" s="10" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A297" s="10" t="s">
+        <v>825</v>
+      </c>
+      <c r="B297" s="10" t="s">
+        <v>826</v>
+      </c>
+      <c r="C297" s="10" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A298" s="10" t="s">
+        <v>828</v>
+      </c>
+      <c r="B298" s="10" t="s">
+        <v>829</v>
+      </c>
+      <c r="C298" s="10" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A299" s="10" t="s">
+        <v>831</v>
+      </c>
+      <c r="B299" s="10" t="s">
+        <v>832</v>
+      </c>
+      <c r="C299" s="10" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A300" s="10" t="s">
+        <v>834</v>
+      </c>
+      <c r="B300" s="10" t="s">
+        <v>835</v>
+      </c>
+      <c r="C300" s="10" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A301" s="10" t="s">
+        <v>837</v>
+      </c>
+      <c r="B301" s="10" t="s">
+        <v>838</v>
+      </c>
+      <c r="C301" s="10" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A302" s="10" t="s">
+        <v>840</v>
+      </c>
+      <c r="B302" s="10" t="s">
+        <v>841</v>
+      </c>
+      <c r="C302" s="10" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A303" s="10" t="s">
+        <v>843</v>
+      </c>
+      <c r="B303" s="10" t="s">
+        <v>844</v>
+      </c>
+      <c r="C303" s="10" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A304" s="10" t="s">
+        <v>846</v>
+      </c>
+      <c r="B304" s="10" t="s">
+        <v>847</v>
+      </c>
+      <c r="C304" s="10" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A305" s="10" t="s">
+        <v>849</v>
+      </c>
+      <c r="B305" s="10" t="s">
+        <v>850</v>
+      </c>
+      <c r="C305" s="10" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A306" s="10" t="s">
+        <v>852</v>
+      </c>
+      <c r="B306" s="10" t="s">
+        <v>853</v>
+      </c>
+      <c r="C306" s="10" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A307" s="10" t="s">
+        <v>855</v>
+      </c>
+      <c r="B307" s="10" t="s">
+        <v>856</v>
+      </c>
+      <c r="C307" s="10" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A308" s="10" t="s">
+        <v>858</v>
+      </c>
+      <c r="B308" s="10" t="s">
+        <v>859</v>
+      </c>
+      <c r="C308" s="10" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A309" s="10" t="s">
+        <v>861</v>
+      </c>
+      <c r="B309" s="10" t="s">
+        <v>862</v>
+      </c>
+      <c r="C309" s="10" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A310" s="10" t="s">
+        <v>864</v>
+      </c>
+      <c r="B310" s="10" t="s">
+        <v>865</v>
+      </c>
+      <c r="C310" s="10" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A311" s="10" t="s">
+        <v>867</v>
+      </c>
+      <c r="B311" s="10" t="s">
+        <v>868</v>
+      </c>
+      <c r="C311" s="10" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A312" s="10" t="s">
+        <v>870</v>
+      </c>
+      <c r="B312" s="10" t="s">
+        <v>871</v>
+      </c>
+      <c r="C312" s="10" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A313" s="10" t="s">
+        <v>873</v>
+      </c>
+      <c r="B313" s="10" t="s">
+        <v>874</v>
+      </c>
+      <c r="C313" s="10" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A314" s="10" t="s">
+        <v>876</v>
+      </c>
+      <c r="B314" s="10" t="s">
+        <v>877</v>
+      </c>
+      <c r="C314" s="10" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A315" s="10" t="s">
         <v>879</v>
       </c>
-      <c r="B293" s="10" t="s">
+      <c r="B315" s="10" t="s">
         <v>880</v>
       </c>
-      <c r="C293" s="10" t="s">
+      <c r="C315" s="10" t="s">
         <v>881</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C21">
-    <sortCondition ref="A2:A21"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C43">
+    <sortCondition ref="A43"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="C38" r:id="rId1" xr:uid="{22C4024E-F5EE-4C14-B35D-9A99EB6AF0F4}"/>
+    <hyperlink ref="C60" r:id="rId1" xr:uid="{22C4024E-F5EE-4C14-B35D-9A99EB6AF0F4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added bycatch text for Azores region
</commit_message>
<xml_diff>
--- a/data-raw/texts.xlsx
+++ b/data-raw/texts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub_2023\fisheriesXplorer\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sarah.weisberg\fisheriesXplorer\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9AFCFF6-EC9A-4DDE-BDB7-11F2F00078F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC39F11-6744-43EE-8C70-20B31016904C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="826" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-50820" yWindow="-4785" windowWidth="40050" windowHeight="15105" tabRatio="858" firstSheet="30" activeTab="48" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="glossary" sheetId="17" r:id="rId1"/>
@@ -59,7 +59,9 @@
     <sheet name="vms_NwS" sheetId="46" r:id="rId44"/>
     <sheet name="vms_ONA" sheetId="47" r:id="rId45"/>
     <sheet name="mixfish" sheetId="5" r:id="rId46"/>
-    <sheet name="bycatch" sheetId="7" r:id="rId47"/>
+    <sheet name="Sheet1" sheetId="48" r:id="rId47"/>
+    <sheet name="bycatch" sheetId="7" r:id="rId48"/>
+    <sheet name="bycatch_AZ" sheetId="49" r:id="rId49"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -82,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1247" uniqueCount="997">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="1001">
   <si>
     <t>section</t>
   </si>
@@ -4717,6 +4719,32 @@
   </si>
   <si>
     <t>https://vocab.ices.dk/?codeguid=023236fc-b701-40b1-90d5-4d09ff60764c</t>
+  </si>
+  <si>
+    <t>total_bycatch</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt;Bycatch of endangered, threatened and protected species&lt;/h4&gt;
+&lt;p&gt;
+All fisheries have the potential to catch endangered, protected and threatened (ETP) species as non-targeted bycatch. The list of ETP marine mammal, seabird, fish and marine turtle species of bycatch relevance for the Azores ecoregion can be found in &lt;a href = "https://doi.org/10.17895/ices.pub.31245037" target = "_blank"&gt;  ICES Roadmap &lt;/a&gt;. For 2024 ICES provides bycatch estimates on marine turtles and multiannual bycatch rates for marine mammals and marine turtles. Due to data limitation ICES estimates bycatch only for certain species and métier combinations.  See&lt;a href = "https://doi.org/10.17895/ices.advice.30734714" target = "_blank"&gt;  ICES (2025) &lt;/a&gt; for more details
+&lt;/p&gt; 
+&lt;h4&gt;Bycatch estimates&lt;/h4&gt;
+&lt;p&gt;
+Total bycatch numbers were estimated for 2 marine turtle species (3 métier/species combinations). The highest total bycaught number was estimated for loggerhead turtle in set gillnet followed by loggerhead turtle in drifting longlines and leatherback turtle in drifting longlines.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>bpue</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt;Bycatch of endangered, threatened and protected species&lt;/h4&gt;
+&lt;p&gt;
+All fisheries have the potential to catch endangered, protected and threatened (ETP) species as non-targeted bycatch. The list of ETP marine mammal, seabird, fish and marine turtle species of bycatch relevance for the Azores ecoregion can be found in &lt;a href = "https://doi.org/10.17895/ices.pub.31245037" target = "_blank"&gt;  ICES Roadmap &lt;/a&gt;. For 2024 ICES provides bycatch estimates on marine turtles and multiannual bycatch rates for marine mammals and marine turtles. Due to data limitation ICES estimates bycatch only for certain species and métier combinations.  See&lt;a href = "https://doi.org/10.17895/ices.advice.30734714" target = "_blank"&gt;  ICES (2025) &lt;/a&gt; for more details
+&lt;/p&gt; 
+&lt;h4&gt;Bycatch rate estimates&lt;/h4&gt;
+&lt;p&gt;
+Multiannual bycatch rates were estimated for 2 marine mammal species (3 métier/species combinations). The highest bycatch rate was estimated for Atlantic spotted dolphin in hand and pole lines, followed by common dolphin in hand and pole lines (mechanized) and hand and pole lines. &lt;/p&gt;
+&lt;p&gt;
+Multiannual bycatch rates were estimated for 3 marine turtle species (4 métier/species combinations). The highest bycatch rate was estimated for loggerhead turtle in drifting longlines, followed by loggerhead turtle in set gillnet and leatherback turtle in drifting longlines.&lt;/p&gt;</t>
   </si>
 </sst>
 </file>
@@ -5154,16 +5182,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF5EC4FE-E411-4E36-B8C3-47DB4028DB0F}">
   <dimension ref="A1:C314"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="168.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="29.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="37.6640625" customWidth="1"/>
-    <col min="17" max="17" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="168.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="29.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="37.7109375" customWidth="1"/>
+    <col min="17" max="17" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -5174,7 +5202,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>29</v>
       </c>
@@ -5185,7 +5213,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>43</v>
       </c>
@@ -5196,7 +5224,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>15</v>
       </c>
@@ -5207,7 +5235,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>20</v>
       </c>
@@ -5218,7 +5246,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>931</v>
       </c>
@@ -5229,7 +5257,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>45</v>
       </c>
@@ -5240,7 +5268,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>21</v>
       </c>
@@ -5251,7 +5279,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>13</v>
       </c>
@@ -5262,7 +5290,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>25</v>
       </c>
@@ -5273,7 +5301,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>934</v>
       </c>
@@ -5284,7 +5312,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>937</v>
       </c>
@@ -5295,7 +5323,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>940</v>
       </c>
@@ -5306,7 +5334,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>943</v>
       </c>
@@ -5317,7 +5345,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>946</v>
       </c>
@@ -5328,7 +5356,7 @@
         <v>948</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>949</v>
       </c>
@@ -5339,7 +5367,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>952</v>
       </c>
@@ -5350,7 +5378,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>49</v>
       </c>
@@ -5361,7 +5389,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>18</v>
       </c>
@@ -5372,7 +5400,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>955</v>
       </c>
@@ -5383,7 +5411,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>958</v>
       </c>
@@ -5394,7 +5422,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>961</v>
       </c>
@@ -5405,7 +5433,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>964</v>
       </c>
@@ -5416,7 +5444,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>41</v>
       </c>
@@ -5427,7 +5455,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>967</v>
       </c>
@@ -5438,7 +5466,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>23</v>
       </c>
@@ -5449,7 +5477,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
         <v>35</v>
       </c>
@@ -5460,7 +5488,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>31</v>
       </c>
@@ -5471,7 +5499,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>27</v>
       </c>
@@ -5482,7 +5510,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>970</v>
       </c>
@@ -5493,7 +5521,7 @@
         <v>972</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>973</v>
       </c>
@@ -5504,7 +5532,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>976</v>
       </c>
@@ -5515,7 +5543,7 @@
         <v>978</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>979</v>
       </c>
@@ -5526,7 +5554,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>982</v>
       </c>
@@ -5537,7 +5565,7 @@
         <v>984</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>985</v>
       </c>
@@ -5548,7 +5576,7 @@
         <v>987</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>988</v>
       </c>
@@ -5559,7 +5587,7 @@
         <v>990</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>991</v>
       </c>
@@ -5570,7 +5598,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>39</v>
       </c>
@@ -5581,7 +5609,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>994</v>
       </c>
@@ -5592,7 +5620,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
         <v>33</v>
       </c>
@@ -5603,7 +5631,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
         <v>37</v>
       </c>
@@ -5614,7 +5642,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
         <v>47</v>
       </c>
@@ -5625,7 +5653,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
         <v>66</v>
       </c>
@@ -5636,7 +5664,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
         <v>69</v>
       </c>
@@ -5647,7 +5675,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
         <v>72</v>
       </c>
@@ -5658,7 +5686,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
         <v>75</v>
       </c>
@@ -5669,7 +5697,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
         <v>78</v>
       </c>
@@ -5680,7 +5708,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
         <v>81</v>
       </c>
@@ -5691,7 +5719,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
         <v>84</v>
       </c>
@@ -5702,7 +5730,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
         <v>87</v>
       </c>
@@ -5713,7 +5741,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
         <v>90</v>
       </c>
@@ -5724,7 +5752,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
         <v>93</v>
       </c>
@@ -5735,7 +5763,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
         <v>96</v>
       </c>
@@ -5746,7 +5774,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
         <v>99</v>
       </c>
@@ -5757,7 +5785,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
         <v>102</v>
       </c>
@@ -5768,7 +5796,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
         <v>105</v>
       </c>
@@ -5779,7 +5807,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>108</v>
       </c>
@@ -5790,7 +5818,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>111</v>
       </c>
@@ -5801,7 +5829,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
         <v>114</v>
       </c>
@@ -5812,7 +5840,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
         <v>117</v>
       </c>
@@ -5823,7 +5851,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="10" t="s">
         <v>120</v>
       </c>
@@ -5834,7 +5862,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
         <v>123</v>
       </c>
@@ -5845,7 +5873,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
         <v>126</v>
       </c>
@@ -5856,7 +5884,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
         <v>129</v>
       </c>
@@ -5867,7 +5895,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="10" t="s">
         <v>132</v>
       </c>
@@ -5878,7 +5906,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
         <v>135</v>
       </c>
@@ -5889,7 +5917,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="10" t="s">
         <v>138</v>
       </c>
@@ -5900,7 +5928,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
         <v>141</v>
       </c>
@@ -5911,7 +5939,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
         <v>144</v>
       </c>
@@ -5922,7 +5950,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
         <v>147</v>
       </c>
@@ -5933,7 +5961,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="10" t="s">
         <v>150</v>
       </c>
@@ -5944,7 +5972,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
         <v>153</v>
       </c>
@@ -5955,7 +5983,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="10" t="s">
         <v>156</v>
       </c>
@@ -5966,7 +5994,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
         <v>159</v>
       </c>
@@ -5977,7 +6005,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
         <v>162</v>
       </c>
@@ -5988,7 +6016,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
         <v>165</v>
       </c>
@@ -5999,7 +6027,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="10" t="s">
         <v>168</v>
       </c>
@@ -6010,7 +6038,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
         <v>171</v>
       </c>
@@ -6021,7 +6049,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="10" t="s">
         <v>174</v>
       </c>
@@ -6032,7 +6060,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
         <v>177</v>
       </c>
@@ -6043,7 +6071,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="10" t="s">
         <v>180</v>
       </c>
@@ -6054,7 +6082,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
         <v>183</v>
       </c>
@@ -6065,7 +6093,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
         <v>186</v>
       </c>
@@ -6076,7 +6104,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
         <v>189</v>
       </c>
@@ -6087,7 +6115,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="10" t="s">
         <v>192</v>
       </c>
@@ -6098,7 +6126,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="10" t="s">
         <v>195</v>
       </c>
@@ -6109,7 +6137,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="10" t="s">
         <v>198</v>
       </c>
@@ -6120,7 +6148,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="10" t="s">
         <v>201</v>
       </c>
@@ -6131,7 +6159,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="10" t="s">
         <v>204</v>
       </c>
@@ -6142,7 +6170,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="10" t="s">
         <v>207</v>
       </c>
@@ -6153,7 +6181,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="10" t="s">
         <v>210</v>
       </c>
@@ -6164,7 +6192,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="10" t="s">
         <v>213</v>
       </c>
@@ -6175,7 +6203,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="10" t="s">
         <v>216</v>
       </c>
@@ -6186,7 +6214,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="10" t="s">
         <v>219</v>
       </c>
@@ -6197,7 +6225,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="10" t="s">
         <v>222</v>
       </c>
@@ -6208,7 +6236,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="10" t="s">
         <v>225</v>
       </c>
@@ -6219,7 +6247,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="10" t="s">
         <v>228</v>
       </c>
@@ -6230,7 +6258,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" s="10" t="s">
         <v>231</v>
       </c>
@@ -6241,7 +6269,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" s="10" t="s">
         <v>234</v>
       </c>
@@ -6252,7 +6280,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" s="10" t="s">
         <v>237</v>
       </c>
@@ -6263,7 +6291,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="10" t="s">
         <v>240</v>
       </c>
@@ -6274,7 +6302,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="10" t="s">
         <v>243</v>
       </c>
@@ -6285,7 +6313,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="10" t="s">
         <v>246</v>
       </c>
@@ -6296,7 +6324,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="10" t="s">
         <v>249</v>
       </c>
@@ -6307,7 +6335,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" s="10" t="s">
         <v>252</v>
       </c>
@@ -6318,7 +6346,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" s="10" t="s">
         <v>255</v>
       </c>
@@ -6329,7 +6357,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" s="10" t="s">
         <v>258</v>
       </c>
@@ -6340,7 +6368,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" s="10" t="s">
         <v>261</v>
       </c>
@@ -6351,7 +6379,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" s="10" t="s">
         <v>264</v>
       </c>
@@ -6362,7 +6390,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" s="10" t="s">
         <v>267</v>
       </c>
@@ -6373,7 +6401,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" s="10" t="s">
         <v>270</v>
       </c>
@@ -6384,7 +6412,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" s="10" t="s">
         <v>273</v>
       </c>
@@ -6395,7 +6423,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="10" t="s">
         <v>276</v>
       </c>
@@ -6406,7 +6434,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" s="10" t="s">
         <v>279</v>
       </c>
@@ -6417,7 +6445,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="10" t="s">
         <v>282</v>
       </c>
@@ -6428,7 +6456,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="10" t="s">
         <v>285</v>
       </c>
@@ -6439,7 +6467,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="10" t="s">
         <v>288</v>
       </c>
@@ -6450,7 +6478,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="10" t="s">
         <v>291</v>
       </c>
@@ -6461,7 +6489,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
         <v>294</v>
       </c>
@@ -6472,7 +6500,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="10" t="s">
         <v>297</v>
       </c>
@@ -6483,7 +6511,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" s="10" t="s">
         <v>300</v>
       </c>
@@ -6494,7 +6522,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" s="10" t="s">
         <v>303</v>
       </c>
@@ -6505,7 +6533,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" s="10" t="s">
         <v>306</v>
       </c>
@@ -6516,7 +6544,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" s="10" t="s">
         <v>309</v>
       </c>
@@ -6527,7 +6555,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" s="10" t="s">
         <v>312</v>
       </c>
@@ -6538,7 +6566,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="10" t="s">
         <v>315</v>
       </c>
@@ -6549,7 +6577,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" s="10" t="s">
         <v>318</v>
       </c>
@@ -6560,7 +6588,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" s="10" t="s">
         <v>321</v>
       </c>
@@ -6571,7 +6599,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="10" t="s">
         <v>324</v>
       </c>
@@ -6582,7 +6610,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="10" t="s">
         <v>327</v>
       </c>
@@ -6593,7 +6621,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="10" t="s">
         <v>330</v>
       </c>
@@ -6604,7 +6632,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" s="10" t="s">
         <v>333</v>
       </c>
@@ -6615,7 +6643,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" s="10" t="s">
         <v>336</v>
       </c>
@@ -6626,7 +6654,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" s="10" t="s">
         <v>339</v>
       </c>
@@ -6637,7 +6665,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" s="10" t="s">
         <v>342</v>
       </c>
@@ -6648,7 +6676,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" s="10" t="s">
         <v>345</v>
       </c>
@@ -6659,7 +6687,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" s="10" t="s">
         <v>348</v>
       </c>
@@ -6670,7 +6698,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" s="10" t="s">
         <v>351</v>
       </c>
@@ -6681,7 +6709,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" s="10" t="s">
         <v>354</v>
       </c>
@@ -6692,7 +6720,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" s="10" t="s">
         <v>357</v>
       </c>
@@ -6703,7 +6731,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" s="10" t="s">
         <v>360</v>
       </c>
@@ -6714,7 +6742,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" s="10" t="s">
         <v>363</v>
       </c>
@@ -6725,7 +6753,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" s="10" t="s">
         <v>366</v>
       </c>
@@ -6736,7 +6764,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" s="10" t="s">
         <v>369</v>
       </c>
@@ -6747,7 +6775,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" s="10" t="s">
         <v>372</v>
       </c>
@@ -6758,7 +6786,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" s="10" t="s">
         <v>375</v>
       </c>
@@ -6769,7 +6797,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" s="10" t="s">
         <v>378</v>
       </c>
@@ -6780,7 +6808,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" s="10" t="s">
         <v>381</v>
       </c>
@@ -6791,7 +6819,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" s="10" t="s">
         <v>384</v>
       </c>
@@ -6802,7 +6830,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" s="10" t="s">
         <v>387</v>
       </c>
@@ -6813,7 +6841,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" s="10" t="s">
         <v>390</v>
       </c>
@@ -6824,7 +6852,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" s="10" t="s">
         <v>393</v>
       </c>
@@ -6835,7 +6863,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" s="10" t="s">
         <v>396</v>
       </c>
@@ -6846,7 +6874,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" s="10" t="s">
         <v>399</v>
       </c>
@@ -6857,7 +6885,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" s="10" t="s">
         <v>402</v>
       </c>
@@ -6868,7 +6896,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" s="10" t="s">
         <v>405</v>
       </c>
@@ -6879,7 +6907,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" s="10" t="s">
         <v>408</v>
       </c>
@@ -6890,7 +6918,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" s="10" t="s">
         <v>411</v>
       </c>
@@ -6901,7 +6929,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" s="10" t="s">
         <v>414</v>
       </c>
@@ -6912,7 +6940,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" s="10" t="s">
         <v>417</v>
       </c>
@@ -6923,7 +6951,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" s="10" t="s">
         <v>420</v>
       </c>
@@ -6934,7 +6962,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" s="10" t="s">
         <v>423</v>
       </c>
@@ -6945,7 +6973,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" s="10" t="s">
         <v>426</v>
       </c>
@@ -6956,7 +6984,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" s="10" t="s">
         <v>429</v>
       </c>
@@ -6967,7 +6995,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" s="10" t="s">
         <v>432</v>
       </c>
@@ -6978,7 +7006,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" s="10" t="s">
         <v>435</v>
       </c>
@@ -6989,7 +7017,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" s="10" t="s">
         <v>438</v>
       </c>
@@ -7000,7 +7028,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" s="10" t="s">
         <v>441</v>
       </c>
@@ -7011,7 +7039,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" s="10" t="s">
         <v>444</v>
       </c>
@@ -7022,7 +7050,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" s="10" t="s">
         <v>447</v>
       </c>
@@ -7033,7 +7061,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" s="10" t="s">
         <v>450</v>
       </c>
@@ -7044,7 +7072,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" s="10" t="s">
         <v>453</v>
       </c>
@@ -7055,7 +7083,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" s="10" t="s">
         <v>456</v>
       </c>
@@ -7066,7 +7094,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" s="10" t="s">
         <v>459</v>
       </c>
@@ -7077,7 +7105,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" s="10" t="s">
         <v>462</v>
       </c>
@@ -7088,7 +7116,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" s="10" t="s">
         <v>465</v>
       </c>
@@ -7099,7 +7127,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="10" t="s">
         <v>468</v>
       </c>
@@ -7110,7 +7138,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="10" t="s">
         <v>471</v>
       </c>
@@ -7121,7 +7149,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="10" t="s">
         <v>474</v>
       </c>
@@ -7132,7 +7160,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="10" t="s">
         <v>477</v>
       </c>
@@ -7143,7 +7171,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="10" t="s">
         <v>480</v>
       </c>
@@ -7154,7 +7182,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="10" t="s">
         <v>483</v>
       </c>
@@ -7165,7 +7193,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="10" t="s">
         <v>486</v>
       </c>
@@ -7176,7 +7204,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="10" t="s">
         <v>489</v>
       </c>
@@ -7187,7 +7215,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="10" t="s">
         <v>492</v>
       </c>
@@ -7198,7 +7226,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="10" t="s">
         <v>495</v>
       </c>
@@ -7209,7 +7237,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="10" t="s">
         <v>498</v>
       </c>
@@ -7220,7 +7248,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="10" t="s">
         <v>501</v>
       </c>
@@ -7231,7 +7259,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="10" t="s">
         <v>504</v>
       </c>
@@ -7242,7 +7270,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="10" t="s">
         <v>507</v>
       </c>
@@ -7253,7 +7281,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="10" t="s">
         <v>510</v>
       </c>
@@ -7264,7 +7292,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="10" t="s">
         <v>513</v>
       </c>
@@ -7275,7 +7303,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="10" t="s">
         <v>516</v>
       </c>
@@ -7286,7 +7314,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="10" t="s">
         <v>519</v>
       </c>
@@ -7297,7 +7325,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="10" t="s">
         <v>522</v>
       </c>
@@ -7308,7 +7336,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="10" t="s">
         <v>525</v>
       </c>
@@ -7319,7 +7347,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="10" t="s">
         <v>528</v>
       </c>
@@ -7330,7 +7358,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="10" t="s">
         <v>531</v>
       </c>
@@ -7341,7 +7369,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="10" t="s">
         <v>534</v>
       </c>
@@ -7352,7 +7380,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="10" t="s">
         <v>537</v>
       </c>
@@ -7363,7 +7391,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="10" t="s">
         <v>540</v>
       </c>
@@ -7374,7 +7402,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="10" t="s">
         <v>543</v>
       </c>
@@ -7385,7 +7413,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="10" t="s">
         <v>546</v>
       </c>
@@ -7396,7 +7424,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="10" t="s">
         <v>549</v>
       </c>
@@ -7407,7 +7435,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="10" t="s">
         <v>552</v>
       </c>
@@ -7418,7 +7446,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="10" t="s">
         <v>555</v>
       </c>
@@ -7429,7 +7457,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="10" t="s">
         <v>558</v>
       </c>
@@ -7440,7 +7468,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" s="10" t="s">
         <v>561</v>
       </c>
@@ -7451,7 +7479,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" s="10" t="s">
         <v>564</v>
       </c>
@@ -7462,7 +7490,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" s="10" t="s">
         <v>567</v>
       </c>
@@ -7473,7 +7501,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" s="10" t="s">
         <v>570</v>
       </c>
@@ -7484,7 +7512,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" s="10" t="s">
         <v>573</v>
       </c>
@@ -7495,7 +7523,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" s="10" t="s">
         <v>576</v>
       </c>
@@ -7506,7 +7534,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" s="10" t="s">
         <v>579</v>
       </c>
@@ -7517,7 +7545,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" s="10" t="s">
         <v>582</v>
       </c>
@@ -7528,7 +7556,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" s="10" t="s">
         <v>585</v>
       </c>
@@ -7539,7 +7567,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" s="10" t="s">
         <v>588</v>
       </c>
@@ -7550,7 +7578,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" s="10" t="s">
         <v>591</v>
       </c>
@@ -7561,7 +7589,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" s="10" t="s">
         <v>594</v>
       </c>
@@ -7572,7 +7600,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" s="10" t="s">
         <v>597</v>
       </c>
@@ -7583,7 +7611,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" s="10" t="s">
         <v>600</v>
       </c>
@@ -7594,7 +7622,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" s="10" t="s">
         <v>603</v>
       </c>
@@ -7605,7 +7633,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" s="10" t="s">
         <v>606</v>
       </c>
@@ -7616,7 +7644,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" s="10" t="s">
         <v>609</v>
       </c>
@@ -7627,7 +7655,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" s="10" t="s">
         <v>612</v>
       </c>
@@ -7638,7 +7666,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" s="10" t="s">
         <v>615</v>
       </c>
@@ -7649,7 +7677,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" s="10" t="s">
         <v>618</v>
       </c>
@@ -7660,7 +7688,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" s="10" t="s">
         <v>621</v>
       </c>
@@ -7671,7 +7699,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" s="10" t="s">
         <v>624</v>
       </c>
@@ -7682,7 +7710,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" s="10" t="s">
         <v>627</v>
       </c>
@@ -7693,7 +7721,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="10" t="s">
         <v>630</v>
       </c>
@@ -7704,7 +7732,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" s="10" t="s">
         <v>633</v>
       </c>
@@ -7715,7 +7743,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" s="10" t="s">
         <v>636</v>
       </c>
@@ -7726,7 +7754,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" s="10" t="s">
         <v>639</v>
       </c>
@@ -7737,7 +7765,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" s="10" t="s">
         <v>642</v>
       </c>
@@ -7748,7 +7776,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="10" t="s">
         <v>645</v>
       </c>
@@ -7759,7 +7787,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" s="10" t="s">
         <v>648</v>
       </c>
@@ -7770,7 +7798,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" s="10" t="s">
         <v>651</v>
       </c>
@@ -7781,7 +7809,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" s="10" t="s">
         <v>654</v>
       </c>
@@ -7792,7 +7820,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" s="10" t="s">
         <v>657</v>
       </c>
@@ -7803,7 +7831,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" s="10" t="s">
         <v>660</v>
       </c>
@@ -7814,7 +7842,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" s="10" t="s">
         <v>663</v>
       </c>
@@ -7825,7 +7853,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" s="10" t="s">
         <v>666</v>
       </c>
@@ -7836,7 +7864,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" s="10" t="s">
         <v>669</v>
       </c>
@@ -7847,7 +7875,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" s="10" t="s">
         <v>672</v>
       </c>
@@ -7858,7 +7886,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" s="10" t="s">
         <v>675</v>
       </c>
@@ -7869,7 +7897,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="10" t="s">
         <v>678</v>
       </c>
@@ -7880,7 +7908,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" s="10" t="s">
         <v>681</v>
       </c>
@@ -7891,7 +7919,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" s="10" t="s">
         <v>684</v>
       </c>
@@ -7902,7 +7930,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250" s="10" t="s">
         <v>687</v>
       </c>
@@ -7913,7 +7941,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" s="10" t="s">
         <v>690</v>
       </c>
@@ -7924,7 +7952,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" s="10" t="s">
         <v>693</v>
       </c>
@@ -7935,7 +7963,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="253" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" s="10" t="s">
         <v>696</v>
       </c>
@@ -7946,7 +7974,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" s="10" t="s">
         <v>699</v>
       </c>
@@ -7957,7 +7985,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" s="10" t="s">
         <v>702</v>
       </c>
@@ -7968,7 +7996,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" s="10" t="s">
         <v>705</v>
       </c>
@@ -7979,7 +8007,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" s="10" t="s">
         <v>708</v>
       </c>
@@ -7990,7 +8018,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="258" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" s="10" t="s">
         <v>711</v>
       </c>
@@ -8001,7 +8029,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" s="10" t="s">
         <v>714</v>
       </c>
@@ -8012,7 +8040,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" s="10" t="s">
         <v>717</v>
       </c>
@@ -8023,7 +8051,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" s="10" t="s">
         <v>720</v>
       </c>
@@ -8034,7 +8062,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" s="10" t="s">
         <v>723</v>
       </c>
@@ -8045,7 +8073,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" s="10" t="s">
         <v>726</v>
       </c>
@@ -8056,7 +8084,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" s="10" t="s">
         <v>729</v>
       </c>
@@ -8067,7 +8095,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265" s="10" t="s">
         <v>732</v>
       </c>
@@ -8078,7 +8106,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" s="10" t="s">
         <v>735</v>
       </c>
@@ -8089,7 +8117,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" s="10" t="s">
         <v>738</v>
       </c>
@@ -8100,7 +8128,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" s="10" t="s">
         <v>741</v>
       </c>
@@ -8111,7 +8139,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A269" s="10" t="s">
         <v>744</v>
       </c>
@@ -8122,7 +8150,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" s="10" t="s">
         <v>747</v>
       </c>
@@ -8133,7 +8161,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" s="10" t="s">
         <v>750</v>
       </c>
@@ -8144,7 +8172,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" s="10" t="s">
         <v>753</v>
       </c>
@@ -8155,7 +8183,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273" s="10" t="s">
         <v>756</v>
       </c>
@@ -8166,7 +8194,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" s="10" t="s">
         <v>759</v>
       </c>
@@ -8177,7 +8205,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="275" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" s="10" t="s">
         <v>762</v>
       </c>
@@ -8188,7 +8216,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" s="10" t="s">
         <v>765</v>
       </c>
@@ -8199,7 +8227,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="277" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" s="10" t="s">
         <v>768</v>
       </c>
@@ -8210,7 +8238,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" s="10" t="s">
         <v>771</v>
       </c>
@@ -8221,7 +8249,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279" s="10" t="s">
         <v>774</v>
       </c>
@@ -8232,7 +8260,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" s="10" t="s">
         <v>777</v>
       </c>
@@ -8243,7 +8271,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" s="10" t="s">
         <v>780</v>
       </c>
@@ -8254,7 +8282,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" s="10" t="s">
         <v>783</v>
       </c>
@@ -8265,7 +8293,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="283" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" s="10" t="s">
         <v>786</v>
       </c>
@@ -8276,7 +8304,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="284" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" s="10" t="s">
         <v>789</v>
       </c>
@@ -8287,7 +8315,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="285" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" s="10" t="s">
         <v>792</v>
       </c>
@@ -8298,7 +8326,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="286" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" s="10" t="s">
         <v>795</v>
       </c>
@@ -8309,7 +8337,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="287" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287" s="10" t="s">
         <v>798</v>
       </c>
@@ -8320,7 +8348,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A288" s="10" t="s">
         <v>801</v>
       </c>
@@ -8331,7 +8359,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="289" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A289" s="10" t="s">
         <v>804</v>
       </c>
@@ -8342,7 +8370,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A290" s="10" t="s">
         <v>807</v>
       </c>
@@ -8353,7 +8381,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A291" s="10" t="s">
         <v>810</v>
       </c>
@@ -8364,7 +8392,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="292" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A292" s="10" t="s">
         <v>813</v>
       </c>
@@ -8375,7 +8403,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="293" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A293" s="10" t="s">
         <v>816</v>
       </c>
@@ -8386,7 +8414,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="294" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A294" s="10" t="s">
         <v>819</v>
       </c>
@@ -8397,7 +8425,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="295" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295" s="10" t="s">
         <v>822</v>
       </c>
@@ -8408,7 +8436,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="296" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A296" s="10" t="s">
         <v>825</v>
       </c>
@@ -8419,7 +8447,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="297" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A297" s="10" t="s">
         <v>828</v>
       </c>
@@ -8430,7 +8458,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="298" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298" s="10" t="s">
         <v>831</v>
       </c>
@@ -8441,7 +8469,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="299" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A299" s="10" t="s">
         <v>834</v>
       </c>
@@ -8452,7 +8480,7 @@
         <v>836</v>
       </c>
     </row>
-    <row r="300" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A300" s="10" t="s">
         <v>837</v>
       </c>
@@ -8463,7 +8491,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="301" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A301" s="10" t="s">
         <v>840</v>
       </c>
@@ -8474,7 +8502,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A302" s="10" t="s">
         <v>843</v>
       </c>
@@ -8485,7 +8513,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A303" s="10" t="s">
         <v>846</v>
       </c>
@@ -8496,7 +8524,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A304" s="10" t="s">
         <v>849</v>
       </c>
@@ -8507,7 +8535,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A305" s="10" t="s">
         <v>852</v>
       </c>
@@ -8518,7 +8546,7 @@
         <v>854</v>
       </c>
     </row>
-    <row r="306" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A306" s="10" t="s">
         <v>855</v>
       </c>
@@ -8529,7 +8557,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="307" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307" s="10" t="s">
         <v>858</v>
       </c>
@@ -8540,7 +8568,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A308" s="10" t="s">
         <v>861</v>
       </c>
@@ -8551,7 +8579,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="309" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A309" s="10" t="s">
         <v>864</v>
       </c>
@@ -8562,7 +8590,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="310" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A310" s="10" t="s">
         <v>867</v>
       </c>
@@ -8573,7 +8601,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A311" s="10" t="s">
         <v>870</v>
       </c>
@@ -8584,7 +8612,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A312" s="10" t="s">
         <v>873</v>
       </c>
@@ -8595,7 +8623,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A313" s="10" t="s">
         <v>876</v>
       </c>
@@ -8606,7 +8634,7 @@
         <v>878</v>
       </c>
     </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A314" s="10" t="s">
         <v>879</v>
       </c>
@@ -8634,13 +8662,13 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -8648,7 +8676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="120.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="120.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -8656,7 +8684,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="303" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="303" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -8664,7 +8692,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -8683,13 +8711,13 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="198.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="198.28515625" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -8697,7 +8725,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="343.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="343.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -8705,7 +8733,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -8713,7 +8741,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -8729,13 +8757,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{744F2D0C-79DF-4FE3-924E-E680015F9291}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="229.6640625" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="229.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -8743,7 +8771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -8751,7 +8779,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -8759,7 +8787,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -8775,13 +8803,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F2C24DB-5CFD-48C4-BB67-81838BA61C50}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8789,7 +8817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -8797,7 +8825,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="328.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="328.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -8813,13 +8841,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176BBE4C-C868-422D-A432-89141BF78270}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8827,7 +8855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -8835,7 +8863,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="286.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="286.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -8851,13 +8879,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{537C8D36-44B6-40AB-B2F5-C278C8F38BBE}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8865,7 +8893,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -8873,7 +8901,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="288" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="288" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -8889,13 +8917,13 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1208CFA8-0BD4-4A00-92D8-FF2B69E34213}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8903,7 +8931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -8911,7 +8939,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="294" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="294" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -8927,12 +8955,12 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1D76C43-B7D3-42D3-B057-81CA4865142E}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="125.5546875" customWidth="1"/>
+    <col min="2" max="2" width="125.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8940,7 +8968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="374.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -8948,7 +8976,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="330" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -8964,13 +8992,13 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C668CA08-39B4-442C-BE86-54D5793A9F15}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8978,7 +9006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -8986,7 +9014,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="260.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="260.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -9002,13 +9030,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82938685-CEEB-4659-B68E-B225C7C9053C}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9016,7 +9044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -9024,7 +9052,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="308.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="308.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -9040,13 +9068,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C69BDA-CBD4-4A20-96F1-D4184C7A4A9F}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="152.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="152.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -9054,7 +9082,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="258.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="258.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -9062,7 +9090,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -9070,7 +9098,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="144" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -9086,13 +9114,13 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED2B002E-5D4B-4A97-8E05-ADA2BC7262BC}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9100,7 +9128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -9108,7 +9136,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="348" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="348" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -9127,13 +9155,13 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9141,7 +9169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -9149,7 +9177,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="244.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="244.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -9165,13 +9193,13 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35913B4E-3457-4352-AB64-7123F047E008}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9179,7 +9207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -9187,7 +9215,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="243.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="243.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -9203,13 +9231,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95FEA048-930A-43AC-A2F7-E864F3A29AEA}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9217,7 +9245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -9225,7 +9253,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="276" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="276" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -9242,13 +9270,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EDA5AB7-BD7F-4972-B610-8565F27586E1}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9256,7 +9284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9264,7 +9292,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9272,7 +9300,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9280,7 +9308,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9294,13 +9322,13 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F3A9AAE-7632-44EA-B097-966294B825CF}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9308,7 +9336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9316,7 +9344,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9324,7 +9352,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9332,7 +9360,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9345,13 +9373,13 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6950BB04-C139-4D8C-A7DF-A5C6DE881B95}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9359,7 +9387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9367,7 +9395,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9375,7 +9403,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9383,7 +9411,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9396,13 +9424,13 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E0EDBDB-CFB0-452E-9EB1-4612E534D157}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9410,7 +9438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9418,7 +9446,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9426,7 +9454,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9434,7 +9462,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9450,13 +9478,13 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9464,7 +9492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9472,7 +9500,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9480,7 +9508,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9488,7 +9516,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9501,13 +9529,13 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BFB3DE4-9A8D-444C-8A7F-95843C784F87}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9515,7 +9543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9523,7 +9551,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9531,7 +9559,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9539,7 +9567,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9552,13 +9580,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58BB4192-B3A0-40C4-9076-17E7860549D0}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="253.88671875" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="253.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -9566,7 +9594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="279" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="279" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -9574,7 +9602,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -9582,7 +9610,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -9598,13 +9626,13 @@
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2C70DEC-BE18-4032-87AC-08A2E40C3A39}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9612,7 +9640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9620,7 +9648,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9628,7 +9656,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9636,7 +9664,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9649,13 +9677,13 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C59D7F3-BDC1-449F-9172-26F24432D1B6}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9663,7 +9691,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9671,7 +9699,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9679,7 +9707,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9687,7 +9715,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9700,13 +9728,13 @@
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AF4D87F-C244-46B9-BEBE-7BAD5D19F1F9}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9714,7 +9742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9722,7 +9750,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9730,7 +9758,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9738,7 +9766,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9751,13 +9779,13 @@
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EFC30CA-8C29-4D4C-B219-684CAC50F683}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9765,7 +9793,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9773,7 +9801,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9781,7 +9809,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9789,7 +9817,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9802,13 +9830,13 @@
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{051B8018-23E1-4D0A-B47D-B5B875F199B2}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="199.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="199.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9816,7 +9844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>884</v>
       </c>
@@ -9824,7 +9852,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>905</v>
       </c>
@@ -9832,7 +9860,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>906</v>
       </c>
@@ -9840,7 +9868,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>907</v>
       </c>
@@ -9856,13 +9884,13 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9870,7 +9898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -9886,13 +9914,13 @@
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CD5BEFF-ABF3-4924-AB24-FF61AF228C0E}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9900,7 +9928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -9916,13 +9944,13 @@
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{924E1A3D-452D-420C-B25E-B5B00D9E4E1C}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9930,7 +9958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -9946,13 +9974,13 @@
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D815AD19-E228-474C-9937-3BF8367B118E}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9960,7 +9988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -9976,13 +10004,13 @@
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D15E140-89C9-45F3-80F4-6B8F3C0CB47C}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9990,7 +10018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -10006,13 +10034,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13D16401-415E-4611-9BEF-C11909718B5A}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="223.88671875" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="223.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -10020,7 +10048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -10028,7 +10056,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -10036,7 +10064,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -10052,13 +10080,13 @@
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DE1070B-144A-405D-8FC5-7DE029CC4010}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10066,7 +10094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -10082,13 +10110,13 @@
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F29691E-1FE6-43C9-8319-10047CCCEDC2}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10096,7 +10124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -10112,13 +10140,13 @@
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44602A52-179B-4771-A428-8A5F60E9F4E5}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10126,7 +10154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -10142,13 +10170,13 @@
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39A8B149-F3B9-47FC-B67F-BAF2CCCF6F3A}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10156,7 +10184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -10172,13 +10200,13 @@
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{407DE1E1-ED4A-4EC4-9635-4F064BD979D5}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10186,7 +10214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -10202,13 +10230,13 @@
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DD0BC59-9F8E-4902-8633-6FC5285FFBA9}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="120.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10216,7 +10244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="271.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>920</v>
       </c>
@@ -10235,12 +10263,12 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10248,7 +10276,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -10262,18 +10290,27 @@
 </file>
 
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E1B14FC-8227-47AA-A858-20FEF7B4AC2B}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="159.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="159.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10281,12 +10318,53 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AE61185-CF8B-43DA-9230-D26A514F1564}">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="120.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="271.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>997</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="285" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>999</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1000</v>
       </c>
     </row>
   </sheetData>
@@ -10297,13 +10375,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA59C6F2-69D0-4598-BA12-1B489ABE98B2}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="181.44140625" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="181.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -10311,7 +10389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -10319,7 +10397,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -10327,7 +10405,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -10343,13 +10421,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBB1D8E1-BE83-467E-ABE2-EB20A46DABB5}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="222.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="222.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -10357,7 +10435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -10365,7 +10443,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -10373,7 +10451,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -10389,13 +10467,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{385D6F23-1F00-43DA-8201-777B854F56F6}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="137.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="137.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -10403,7 +10481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="390" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="393.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -10411,7 +10489,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -10419,7 +10497,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -10427,13 +10505,13 @@
         <v>899</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="5"/>
     </row>
-    <row r="6" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="5"/>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="6"/>
     </row>
   </sheetData>
@@ -10444,13 +10522,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A026B00C-E4B3-4E36-BEA1-AD93DF3D486F}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="135.5546875" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="135.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -10458,7 +10536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -10466,7 +10544,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -10474,7 +10552,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -10490,13 +10568,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27175C00-9C85-488E-AAAE-6AE4E23126BD}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="114.88671875" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="114.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -10504,7 +10582,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>882</v>
       </c>
@@ -10512,7 +10590,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -10520,7 +10598,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
update bycatch API endpoint and refresh text file
</commit_message>
<xml_diff>
--- a/data-raw/texts.xlsx
+++ b/data-raw/texts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub_2023\fisheriesXplorer\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB7F0096-B5B7-4580-8B77-0320AEEE864C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E590FAB-0618-4FA5-B28E-C9CB7538FE79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="858" firstSheet="41" activeTab="45" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="858" firstSheet="41" activeTab="55" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="glossary" sheetId="17" r:id="rId1"/>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1305" uniqueCount="1011">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1305" uniqueCount="1013">
   <si>
     <t>section</t>
   </si>
@@ -4876,6 +4876,26 @@
   </si>
   <si>
     <t>No bycatch advice available for this ecoregion.</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt;Bycatch of endangered, threatened and protected species&lt;/h4&gt;
+&lt;p&gt;
+All fisheries have the potential to catch endangered, protected and threatened (ETP) species as non-targeted bycatch. The list of ETP marine mammal, seabird, fish and marine turtle species of bycatch relevance for the Barents Sea ecoregion can be found in &lt;a href = "https://doi.org/10.17895/ices.pub.31245037" target = "_blank"&gt;  ICES Roadmap &lt;/a&gt;.  For 2024 ICES provides bycatch rate estimates for marine mammals and seabirds. Due to data limitation ICES estimates bycatch only for certain species and métier combinations.  See&lt;a href = "https://doi.org/10.17895/ices.advice.30734714" target = "_blank"&gt;  ICES (2025) &lt;/a&gt; for more details
+&lt;/p&gt;   
+&lt;h4&gt;Bycatch rate estimates&lt;/h4&gt;
+&lt;p&gt;
+Multiannual bycatch rates were estimated for 3 marine mammal species in one métier. The highest bycatch rate was estimated for harbor seal in set gillnets, followed by harbor porpoise in set gillnets and grey seal in set gillnets. &lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt;Bycatch of endangered, threatened and protected species&lt;/h4&gt;
+&lt;p&gt;
+All fisheries have the potential to catch endangered, protected and threatened (ETP) species as non-targeted bycatch. The list of ETP marine mammal, seabird, fish and marine turtle species of bycatch relevance for the Norwegian Sea ecoregion can be found in &lt;a href = "https://doi.org/10.17895/ices.pub.31245037" target = "_blank"&gt;  ICES Roadmap &lt;/a&gt;.  For 2024 ICES provides bycatch estimates on marine mammals and seabirds and bycatch rates for marine mammals and seabirds. Due to data limitation ICES estimates bycatch only for certain species and métier combinations.  See&lt;a href = "https://doi.org/10.17895/ices.advice.30734714" target = "_blank"&gt;  ICES (2025) &lt;/a&gt; for more details
+&lt;/p&gt;   
+&lt;h4&gt;Bycatch rate estimates&lt;/h4&gt;
+&lt;p&gt;
+Multiannual bycatch rates were estimated for 3 marine mammal species in one métier. The highest bycatch rate was estimated for harbor porpoise in set gillnets, followed by harbor seal in set gillnets and grey seal in set gillnets. &lt;/p&gt;
+&lt;p&gt;
+Multiannual bycatch rates were estimated for 5 seabird species in one métier. The highest bycatch rate was estimated for northern fulmar in set gillnets, followed by common guillemot in set gillnets and razorbill in set gillnets.  &lt;/p&gt;</t>
   </si>
 </sst>
 </file>
@@ -10435,7 +10455,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="65.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="109.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -10492,12 +10512,12 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>995</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
     </row>
   </sheetData>
@@ -10803,12 +10823,12 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>995</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1010</v>
+        <v>1012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>